<commit_message>
Dashboard: 2026-07-06 20:32 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1334,6 +1334,43 @@
         </is>
       </c>
       <c r="G24" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06/07/2026 17:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>819</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>6091</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>687</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -4321,7 +4358,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -9262,7 +9299,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -10101,7 +10138,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>92</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -14920,7 +14957,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -18473,7 +18510,7 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>71</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -18577,7 +18614,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -20617,7 +20654,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -27091,7 +27128,7 @@
       </c>
       <c r="F492" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>132</t>
         </is>
       </c>
       <c r="G492" t="inlineStr">
@@ -34034,7 +34071,7 @@
       </c>
       <c r="F625" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G625" t="inlineStr">
@@ -34894,7 +34931,7 @@
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>Atualizado: 03/07/2026 13:08 | Ativas: 819 | Inativas: 0</t>
+          <t>Atualizado: 06/07/2026 17:00 | Ativas: 819 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53310,7 +53347,7 @@
     <row r="690">
       <c r="A690" t="inlineStr">
         <is>
-          <t>Atualizado: 03/07/2026 13:08 | Total: 687 | c/ usuario: 169 | s/ usuario: 518</t>
+          <t>Atualizado: 06/07/2026 17:00 | Total: 687 | c/ usuario: 169 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -53325,7 +53362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C657"/>
+  <dimension ref="A1:C660"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -61846,16 +61883,55 @@
         </is>
       </c>
       <c r="B655" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C655" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>04/07/2026</t>
+        </is>
+      </c>
+      <c r="B656" t="n">
+        <v>6</v>
+      </c>
+      <c r="C656" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 03/07/2026 13:08 | Total dias: 654</t>
+          <t>05/07/2026</t>
+        </is>
+      </c>
+      <c r="B657" t="n">
+        <v>2</v>
+      </c>
+      <c r="C657" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="B658" t="n">
+        <v>5</v>
+      </c>
+      <c r="C658" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Atualizado: 06/07/2026 17:00 | Total dias: 657</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-07 17:39 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1408,6 +1408,43 @@
         </is>
       </c>
       <c r="G26" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07/07/2026 14:36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>6096</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -3665,7 +3702,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -14421,7 +14458,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -27375,7 +27412,7 @@
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G496" t="inlineStr">
@@ -35021,7 +35058,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 09:53 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 07/07/2026 14:36 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53464,7 +53501,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 09:53 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 07/07/2026 14:36 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -53479,7 +53516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C660"/>
+  <dimension ref="A1:C661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62045,10 +62082,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="660">
-      <c r="A660" t="inlineStr">
-        <is>
-          <t>Atualizado: 07/07/2026 09:53 | Total dias: 657</t>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="B659" t="n">
+        <v>4</v>
+      </c>
+      <c r="C659" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Atualizado: 07/07/2026 14:36 | Total dias: 658</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-07 19:19 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1445,6 +1445,43 @@
         </is>
       </c>
       <c r="G27" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07/07/2026 16:16</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>6098</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -12562,7 +12599,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -26889,7 +26926,7 @@
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G486" t="inlineStr">
@@ -35058,7 +35095,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 14:36 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 07/07/2026 16:16 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53501,7 +53538,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 14:36 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 07/07/2026 16:16 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -62089,7 +62126,7 @@
         </is>
       </c>
       <c r="B659" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C659" t="n">
         <v>0</v>
@@ -62098,7 +62135,7 @@
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 14:36 | Total dias: 658</t>
+          <t>Atualizado: 07/07/2026 16:16 | Total dias: 658</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-07 19:26 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1482,6 +1482,43 @@
         </is>
       </c>
       <c r="G28" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07/07/2026 16:23</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6098</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -35095,7 +35132,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 16:16 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 07/07/2026 16:23 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53538,7 +53575,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 16:16 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 07/07/2026 16:23 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -62135,7 +62172,7 @@
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 16:16 | Total dias: 658</t>
+          <t>Atualizado: 07/07/2026 16:23 | Total dias: 658</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-08 16:20 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1519,6 +1519,43 @@
         </is>
       </c>
       <c r="G29" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>08/07/2026 13:17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>6105</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -17141,7 +17178,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -22525,7 +22562,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -35132,7 +35169,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 16:23 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 08/07/2026 13:17 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53575,7 +53612,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 07/07/2026 16:23 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 08/07/2026 13:17 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -53590,7 +53627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C661"/>
+  <dimension ref="A1:C662"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62169,10 +62206,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="661">
-      <c r="A661" t="inlineStr">
-        <is>
-          <t>Atualizado: 07/07/2026 16:23 | Total dias: 658</t>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B660" t="n">
+        <v>7</v>
+      </c>
+      <c r="C660" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Atualizado: 08/07/2026 13:17 | Total dias: 659</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-09 13:43 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1556,6 +1556,43 @@
         </is>
       </c>
       <c r="G30" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>09/07/2026 10:39</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>6113</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -5380,7 +5417,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>371</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -5541,7 +5578,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -8434,7 +8471,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>214</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -25223,7 +25260,7 @@
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G452" t="inlineStr">
@@ -27366,7 +27403,7 @@
       </c>
       <c r="F493" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>133</t>
         </is>
       </c>
       <c r="G493" t="inlineStr">
@@ -35169,7 +35206,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 08/07/2026 13:17 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 09/07/2026 10:39 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53612,7 +53649,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 08/07/2026 13:17 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 09/07/2026 10:39 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -53627,7 +53664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C662"/>
+  <dimension ref="A1:C663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62213,16 +62250,29 @@
         </is>
       </c>
       <c r="B660" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C660" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="662">
-      <c r="A662" t="inlineStr">
-        <is>
-          <t>Atualizado: 08/07/2026 13:17 | Total dias: 659</t>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="B661" t="n">
+        <v>4</v>
+      </c>
+      <c r="C661" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Atualizado: 09/07/2026 10:39 | Total dias: 660</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-09 14:35 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1593,6 +1593,43 @@
         </is>
       </c>
       <c r="G31" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>09/07/2026 11:32</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>6113</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -35206,7 +35243,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 10:39 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 09/07/2026 11:32 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53649,7 +53686,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 10:39 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 09/07/2026 11:32 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -62272,7 +62309,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 10:39 | Total dias: 660</t>
+          <t>Atualizado: 09/07/2026 11:32 | Total dias: 660</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-09 14:43 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1630,6 +1630,43 @@
         </is>
       </c>
       <c r="G32" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>09/07/2026 11:41</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>6113</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -35243,7 +35280,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 11:32 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 09/07/2026 11:41 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53686,7 +53723,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 11:32 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 09/07/2026 11:41 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -62309,7 +62346,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 11:32 | Total dias: 660</t>
+          <t>Atualizado: 09/07/2026 11:41 | Total dias: 660</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-09 14:53 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1667,6 +1667,43 @@
         </is>
       </c>
       <c r="G33" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>09/07/2026 11:50</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>6113</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
         <is>
           <t>518</t>
         </is>
@@ -35280,7 +35317,7 @@
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 11:41 | Ativas: 820 | Inativas: 0</t>
+          <t>Atualizado: 09/07/2026 11:50 | Ativas: 820 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53723,7 +53760,7 @@
     <row r="691">
       <c r="A691" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 11:41 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
+          <t>Atualizado: 09/07/2026 11:50 | Total: 688 | c/ usuario: 170 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -62346,7 +62383,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 11:41 | Total dias: 660</t>
+          <t>Atualizado: 09/07/2026 11:50 | Total dias: 660</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-10 17:13 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1741,6 +1741,43 @@
         </is>
       </c>
       <c r="G35" t="inlineStr">
+        <is>
+          <t>517</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>10/07/2026 14:09</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>819</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>6117</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>686</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
         <is>
           <t>517</t>
         </is>
@@ -2798,7 +2835,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3060,7 +3097,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4050,7 +4087,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8511,7 +8548,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>139</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -10612,7 +10649,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -28859,7 +28896,7 @@
       </c>
       <c r="F518" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G518" t="inlineStr">
@@ -29119,7 +29156,7 @@
       </c>
       <c r="F523" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G523" t="inlineStr">
@@ -33345,7 +33382,7 @@
       </c>
       <c r="F604" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>207</t>
         </is>
       </c>
       <c r="G604" t="inlineStr">
@@ -35302,7 +35339,7 @@
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 14:33 | Ativas: 819 | Inativas: 0</t>
+          <t>Atualizado: 10/07/2026 14:09 | Ativas: 819 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53691,7 +53728,7 @@
     <row r="689">
       <c r="A689" t="inlineStr">
         <is>
-          <t>Atualizado: 09/07/2026 14:33 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
+          <t>Atualizado: 10/07/2026 14:09 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
         </is>
       </c>
     </row>
@@ -53706,7 +53743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C663"/>
+  <dimension ref="A1:C664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62305,16 +62342,29 @@
         </is>
       </c>
       <c r="B661" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C661" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="663">
-      <c r="A663" t="inlineStr">
-        <is>
-          <t>Atualizado: 09/07/2026 14:33 | Total dias: 660</t>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="B662" t="n">
+        <v>3</v>
+      </c>
+      <c r="C662" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Atualizado: 10/07/2026 14:09 | Total dias: 661</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-11 14:41 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1778,6 +1778,43 @@
         </is>
       </c>
       <c r="G36" t="inlineStr">
+        <is>
+          <t>517</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>11/07/2026 11:37</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>819</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>6121</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>686</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>517</t>
         </is>
@@ -3357,7 +3394,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -8548,7 +8585,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>140</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -8656,7 +8693,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>215</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -25289,7 +25326,7 @@
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G449" t="inlineStr">
@@ -35339,7 +35376,7 @@
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>Atualizado: 10/07/2026 14:09 | Ativas: 819 | Inativas: 0</t>
+          <t>Atualizado: 11/07/2026 11:37 | Ativas: 819 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53728,7 +53765,7 @@
     <row r="689">
       <c r="A689" t="inlineStr">
         <is>
-          <t>Atualizado: 10/07/2026 14:09 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
+          <t>Atualizado: 11/07/2026 11:37 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
         </is>
       </c>
     </row>
@@ -53743,7 +53780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C664"/>
+  <dimension ref="A1:C665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62355,16 +62392,29 @@
         </is>
       </c>
       <c r="B662" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C662" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="664">
-      <c r="A664" t="inlineStr">
-        <is>
-          <t>Atualizado: 10/07/2026 14:09 | Total dias: 661</t>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="B663" t="n">
+        <v>2</v>
+      </c>
+      <c r="C663" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Atualizado: 11/07/2026 11:37 | Total dias: 662</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-12 14:44 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1815,6 +1815,43 @@
         </is>
       </c>
       <c r="G37" t="inlineStr">
+        <is>
+          <t>517</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>12/07/2026 11:40</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>819</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>6125</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>686</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>517</t>
         </is>
@@ -10634,7 +10671,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>144</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -15610,7 +15647,7 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
@@ -34098,7 +34135,7 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G617" t="inlineStr">
@@ -35376,7 +35413,7 @@
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>Atualizado: 11/07/2026 11:37 | Ativas: 819 | Inativas: 0</t>
+          <t>Atualizado: 12/07/2026 11:40 | Ativas: 819 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53765,7 +53802,7 @@
     <row r="689">
       <c r="A689" t="inlineStr">
         <is>
-          <t>Atualizado: 11/07/2026 11:37 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
+          <t>Atualizado: 12/07/2026 11:40 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
         </is>
       </c>
     </row>
@@ -62405,7 +62442,7 @@
         </is>
       </c>
       <c r="B663" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C663" t="n">
         <v>0</v>
@@ -62414,7 +62451,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 11/07/2026 11:37 | Total dias: 662</t>
+          <t>Atualizado: 12/07/2026 11:40 | Total dias: 662</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-13 17:41 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1852,6 +1852,43 @@
         </is>
       </c>
       <c r="G38" t="inlineStr">
+        <is>
+          <t>517</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>13/07/2026 14:37</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>819</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>6127</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>686</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
         <is>
           <t>517</t>
         </is>
@@ -8622,7 +8659,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -10619,7 +10656,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -35413,7 +35450,7 @@
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>Atualizado: 12/07/2026 11:40 | Ativas: 819 | Inativas: 0</t>
+          <t>Atualizado: 13/07/2026 14:37 | Ativas: 819 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -53802,7 +53839,7 @@
     <row r="689">
       <c r="A689" t="inlineStr">
         <is>
-          <t>Atualizado: 12/07/2026 11:40 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
+          <t>Atualizado: 13/07/2026 14:37 | Total: 686 | c/ usuario: 169 | s/ usuario: 517</t>
         </is>
       </c>
     </row>
@@ -53817,7 +53854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C665"/>
+  <dimension ref="A1:C666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62448,10 +62485,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="665">
-      <c r="A665" t="inlineStr">
-        <is>
-          <t>Atualizado: 12/07/2026 11:40 | Total dias: 662</t>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+      <c r="B664" t="n">
+        <v>2</v>
+      </c>
+      <c r="C664" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Atualizado: 13/07/2026 14:37 | Total dias: 663</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-15 15:19 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1926,6 +1926,43 @@
         </is>
       </c>
       <c r="G40" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>15/07/2026 12:15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>6140</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>691</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -25904,7 +25941,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
@@ -36058,7 +36095,7 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Atualizado: 14/07/2026 12:16 | Ativas: 831 | Inativas: 0</t>
+          <t>Atualizado: 15/07/2026 12:15 | Ativas: 831 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -54582,7 +54619,7 @@
     <row r="694">
       <c r="A694" t="inlineStr">
         <is>
-          <t>Atualizado: 14/07/2026 12:16 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
+          <t>Atualizado: 15/07/2026 12:15 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -54597,7 +54634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C667"/>
+  <dimension ref="A1:C668"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63248,16 +63285,29 @@
         </is>
       </c>
       <c r="B665" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C665" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="667">
-      <c r="A667" t="inlineStr">
-        <is>
-          <t>Atualizado: 14/07/2026 12:16 | Total dias: 664</t>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
+      <c r="B666" t="n">
+        <v>2</v>
+      </c>
+      <c r="C666" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Atualizado: 15/07/2026 12:15 | Total dias: 665</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-16 15:55 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -1963,6 +1963,43 @@
         </is>
       </c>
       <c r="G41" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16/07/2026 12:51</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>6146</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>691</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -5367,7 +5404,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -7160,7 +7197,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -28136,7 +28173,7 @@
       </c>
       <c r="F500" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>134</t>
         </is>
       </c>
       <c r="G500" t="inlineStr">
@@ -29287,7 +29324,7 @@
       </c>
       <c r="F522" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G522" t="inlineStr">
@@ -36095,7 +36132,7 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Atualizado: 15/07/2026 12:15 | Ativas: 831 | Inativas: 0</t>
+          <t>Atualizado: 16/07/2026 12:51 | Ativas: 831 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -54619,7 +54656,7 @@
     <row r="694">
       <c r="A694" t="inlineStr">
         <is>
-          <t>Atualizado: 15/07/2026 12:15 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
+          <t>Atualizado: 16/07/2026 12:51 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -54634,7 +54671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C668"/>
+  <dimension ref="A1:C669"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63298,16 +63335,29 @@
         </is>
       </c>
       <c r="B666" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C666" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="668">
-      <c r="A668" t="inlineStr">
-        <is>
-          <t>Atualizado: 15/07/2026 12:15 | Total dias: 665</t>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
+      <c r="B667" t="n">
+        <v>5</v>
+      </c>
+      <c r="C667" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Atualizado: 16/07/2026 12:51 | Total dias: 666</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-17 15:06 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2000,6 +2000,43 @@
         </is>
       </c>
       <c r="G42" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17/07/2026 12:02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>6152</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>691</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -8717,7 +8754,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>142</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -10136,7 +10173,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -10397,7 +10434,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -21491,7 +21528,7 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
@@ -33287,7 +33324,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">
@@ -36132,7 +36169,7 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Atualizado: 16/07/2026 12:51 | Ativas: 831 | Inativas: 0</t>
+          <t>Atualizado: 17/07/2026 12:02 | Ativas: 831 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -54656,7 +54693,7 @@
     <row r="694">
       <c r="A694" t="inlineStr">
         <is>
-          <t>Atualizado: 16/07/2026 12:51 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
+          <t>Atualizado: 17/07/2026 12:02 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -54671,7 +54708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C669"/>
+  <dimension ref="A1:C670"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63348,16 +63385,29 @@
         </is>
       </c>
       <c r="B667" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C667" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="669">
-      <c r="A669" t="inlineStr">
-        <is>
-          <t>Atualizado: 16/07/2026 12:51 | Total dias: 666</t>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="B668" t="n">
+        <v>4</v>
+      </c>
+      <c r="C668" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Atualizado: 17/07/2026 12:02 | Total dias: 667</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-18 12:46 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2037,6 +2037,43 @@
         </is>
       </c>
       <c r="G43" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>18/07/2026 09:43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>6156</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>691</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -5861,7 +5898,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>371</t>
+          <t>372</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -9808,7 +9845,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -15413,7 +15450,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -28784,7 +28821,7 @@
       </c>
       <c r="F511" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G511" t="inlineStr">
@@ -36169,7 +36206,7 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Atualizado: 17/07/2026 12:02 | Ativas: 831 | Inativas: 0</t>
+          <t>Atualizado: 18/07/2026 09:43 | Ativas: 831 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -54693,7 +54730,7 @@
     <row r="694">
       <c r="A694" t="inlineStr">
         <is>
-          <t>Atualizado: 17/07/2026 12:02 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
+          <t>Atualizado: 18/07/2026 09:43 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -63398,7 +63435,7 @@
         </is>
       </c>
       <c r="B668" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C668" t="n">
         <v>0</v>
@@ -63407,7 +63444,7 @@
     <row r="670">
       <c r="A670" t="inlineStr">
         <is>
-          <t>Atualizado: 17/07/2026 12:02 | Total dias: 667</t>
+          <t>Atualizado: 18/07/2026 09:43 | Total dias: 667</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-19 14:41 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2074,6 +2074,43 @@
         </is>
       </c>
       <c r="G44" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>19/07/2026 11:38</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>6163</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>691</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -2447,7 +2484,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4801,7 +4838,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -11468,7 +11505,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -24958,7 +24995,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
@@ -35918,7 +35955,7 @@
       </c>
       <c r="F647" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G647" t="inlineStr">
@@ -36206,7 +36243,7 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Atualizado: 18/07/2026 09:43 | Ativas: 831 | Inativas: 0</t>
+          <t>Atualizado: 19/07/2026 11:38 | Ativas: 831 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -54730,7 +54767,7 @@
     <row r="694">
       <c r="A694" t="inlineStr">
         <is>
-          <t>Atualizado: 18/07/2026 09:43 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
+          <t>Atualizado: 19/07/2026 11:38 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -54745,7 +54782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C670"/>
+  <dimension ref="A1:C672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63441,10 +63478,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>18/07/2026</t>
+        </is>
+      </c>
+      <c r="B669" t="n">
+        <v>5</v>
+      </c>
+      <c r="C669" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="670">
       <c r="A670" t="inlineStr">
         <is>
-          <t>Atualizado: 18/07/2026 09:43 | Total dias: 667</t>
+          <t>19/07/2026</t>
+        </is>
+      </c>
+      <c r="B670" t="n">
+        <v>2</v>
+      </c>
+      <c r="C670" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Atualizado: 19/07/2026 11:38 | Total dias: 669</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-20 16:14 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2111,6 +2111,43 @@
         </is>
       </c>
       <c r="G45" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>20/07/2026 13:11</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>831</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>6165</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>692</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -24891,7 +24928,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G435" t="inlineStr">
@@ -36243,7 +36280,7 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Atualizado: 19/07/2026 11:38 | Ativas: 831 | Inativas: 0</t>
+          <t>Atualizado: 20/07/2026 13:11 | Ativas: 831 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -36258,7 +36295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E694"/>
+  <dimension ref="A1:E695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -54764,10 +54801,35 @@
         </is>
       </c>
     </row>
-    <row r="694">
-      <c r="A694" t="inlineStr">
-        <is>
-          <t>Atualizado: 19/07/2026 11:38 | Total: 691 | c/ usuario: 175 | s/ usuario: 516</t>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>951</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Deway tecnologia</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Felipe Cesar / felipe.cesar@deway.com.br</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>TECNOLOGIA</t>
+        </is>
+      </c>
+      <c r="E693" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Atualizado: 20/07/2026 13:11 | Total: 692 | c/ usuario: 176 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -54782,7 +54844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C672"/>
+  <dimension ref="A1:C673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63498,16 +63560,29 @@
         </is>
       </c>
       <c r="B670" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C670" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="672">
-      <c r="A672" t="inlineStr">
-        <is>
-          <t>Atualizado: 19/07/2026 11:38 | Total dias: 669</t>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="B671" t="n">
+        <v>1</v>
+      </c>
+      <c r="C671" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Atualizado: 20/07/2026 13:11 | Total dias: 670</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-21 16:01 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2150,6 +2150,43 @@
       <c r="G46" t="inlineStr">
         <is>
           <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:58</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>832</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>6172</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>693</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>517</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3294,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -26756,7 +26793,7 @@
       </c>
       <c r="F470" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>56</t>
         </is>
       </c>
       <c r="G470" t="inlineStr">
@@ -36280,7 +36317,7 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Atualizado: 20/07/2026 13:11 | Ativas: 831 | Inativas: 0</t>
+          <t>Atualizado: 21/07/2026 12:58 | Ativas: 832 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -36295,7 +36332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E695"/>
+  <dimension ref="A1:E696"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -54826,10 +54863,35 @@
         <v>17</v>
       </c>
     </row>
-    <row r="695">
-      <c r="A695" t="inlineStr">
-        <is>
-          <t>Atualizado: 20/07/2026 13:11 | Total: 692 | c/ usuario: 176 | s/ usuario: 516</t>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>952</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Rooftop Piazza Aldeota</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Nao cadastrado</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>EVENTOS</t>
+        </is>
+      </c>
+      <c r="E694" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Atualizado: 21/07/2026 12:58 | Total: 693 | c/ usuario: 176 | s/ usuario: 517</t>
         </is>
       </c>
     </row>
@@ -54844,7 +54906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C673"/>
+  <dimension ref="A1:C674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63573,16 +63635,29 @@
         </is>
       </c>
       <c r="B671" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C671" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="673">
-      <c r="A673" t="inlineStr">
-        <is>
-          <t>Atualizado: 20/07/2026 13:11 | Total dias: 670</t>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="B672" t="n">
+        <v>5</v>
+      </c>
+      <c r="C672" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Atualizado: 21/07/2026 12:58 | Total dias: 671</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-23 16:12 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2222,6 +2222,43 @@
         </is>
       </c>
       <c r="G48" t="inlineStr">
+        <is>
+          <t>521</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>23/07/2026 13:08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>6189</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
         <is>
           <t>521</t>
         </is>
@@ -6046,7 +6083,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>374</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -9047,7 +9084,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>219</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -16330,7 +16367,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -17580,7 +17617,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -23695,7 +23732,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>60</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -33665,7 +33702,7 @@
       </c>
       <c r="F601" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>63</t>
         </is>
       </c>
       <c r="G601" t="inlineStr">
@@ -36510,7 +36547,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 22/07/2026 12:54 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 23/07/2026 13:08 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55186,7 +55223,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 22/07/2026 12:54 | Total: 697 | c/ usuario: 176 | s/ usuario: 521</t>
+          <t>Atualizado: 23/07/2026 13:08 | Total: 697 | c/ usuario: 176 | s/ usuario: 521</t>
         </is>
       </c>
     </row>
@@ -55201,7 +55238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C675"/>
+  <dimension ref="A1:C676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63956,16 +63993,29 @@
         </is>
       </c>
       <c r="B673" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C673" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="675">
-      <c r="A675" t="inlineStr">
-        <is>
-          <t>Atualizado: 22/07/2026 12:54 | Total dias: 672</t>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
+      <c r="B674" t="n">
+        <v>5</v>
+      </c>
+      <c r="C674" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Atualizado: 23/07/2026 13:08 | Total dias: 673</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-24 15:23 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2259,6 +2259,43 @@
         </is>
       </c>
       <c r="G49" t="inlineStr">
+        <is>
+          <t>521</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>24/07/2026 12:19</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>6193</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
         <is>
           <t>521</t>
         </is>
@@ -17617,7 +17654,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -21906,7 +21943,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>78</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -33702,7 +33739,7 @@
       </c>
       <c r="F601" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>64</t>
         </is>
       </c>
       <c r="G601" t="inlineStr">
@@ -34119,7 +34156,7 @@
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G609" t="inlineStr">
@@ -36547,7 +36584,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 23/07/2026 13:08 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 24/07/2026 12:19 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55223,7 +55260,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 23/07/2026 13:08 | Total: 697 | c/ usuario: 176 | s/ usuario: 521</t>
+          <t>Atualizado: 24/07/2026 12:19 | Total: 697 | c/ usuario: 176 | s/ usuario: 521</t>
         </is>
       </c>
     </row>
@@ -55238,7 +55275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C676"/>
+  <dimension ref="A1:C677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64006,16 +64043,29 @@
         </is>
       </c>
       <c r="B674" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C674" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="676">
-      <c r="A676" t="inlineStr">
-        <is>
-          <t>Atualizado: 23/07/2026 13:08 | Total dias: 673</t>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
+      <c r="B675" t="n">
+        <v>2</v>
+      </c>
+      <c r="C675" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Atualizado: 24/07/2026 12:19 | Total dias: 674</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-25 14:52 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2298,6 +2298,43 @@
       <c r="G50" t="inlineStr">
         <is>
           <t>521</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>25/07/2026 11:48</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>6197</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>519</t>
         </is>
       </c>
     </row>
@@ -4866,7 +4903,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>138</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -7124,7 +7161,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -23665,7 +23702,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -26482,7 +26519,7 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G462" t="inlineStr">
@@ -36584,7 +36621,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 24/07/2026 12:19 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 25/07/2026 11:48 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55143,7 +55180,7 @@
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>Nao cadastrado</t>
+          <t>Helena Bonatto Maia / piazzaaldeota@gmail.com</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
@@ -55193,7 +55230,7 @@
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>Nao cadastrado</t>
+          <t>Leonardo Pereira de Oliveira / atendimento.reflexus@gmail.com</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
@@ -55260,7 +55297,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 24/07/2026 12:19 | Total: 697 | c/ usuario: 176 | s/ usuario: 521</t>
+          <t>Atualizado: 25/07/2026 11:48 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55275,7 +55312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C677"/>
+  <dimension ref="A1:C678"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64056,16 +64093,29 @@
         </is>
       </c>
       <c r="B675" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C675" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="677">
-      <c r="A677" t="inlineStr">
-        <is>
-          <t>Atualizado: 24/07/2026 12:19 | Total dias: 674</t>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="B676" t="n">
+        <v>1</v>
+      </c>
+      <c r="C676" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Atualizado: 25/07/2026 11:48 | Total dias: 675</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-26 14:54 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2333,6 +2333,43 @@
         </is>
       </c>
       <c r="G51" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>26/07/2026 11:50</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>6203</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -2915,7 +2952,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4903,7 +4940,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>140</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -9158,7 +9195,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>220</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -11099,7 +11136,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>145</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -33620,7 +33657,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">
@@ -36621,7 +36658,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 25/07/2026 11:48 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 26/07/2026 11:50 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55297,7 +55334,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 25/07/2026 11:48 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 26/07/2026 11:50 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55312,7 +55349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C678"/>
+  <dimension ref="A1:C679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64106,16 +64143,29 @@
         </is>
       </c>
       <c r="B676" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C676" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="678">
-      <c r="A678" t="inlineStr">
-        <is>
-          <t>Atualizado: 25/07/2026 11:48 | Total dias: 675</t>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="B677" t="n">
+        <v>3</v>
+      </c>
+      <c r="C677" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Atualizado: 26/07/2026 11:50 | Total dias: 676</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-27 17:23 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2370,6 +2370,43 @@
         </is>
       </c>
       <c r="G52" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>27/07/2026 14:14</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>6207</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -16738,7 +16775,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -21701,7 +21738,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -29273,7 +29310,7 @@
       </c>
       <c r="F514" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G514" t="inlineStr">
@@ -36658,7 +36695,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 26/07/2026 11:50 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 27/07/2026 14:14 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55334,7 +55371,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 26/07/2026 11:50 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 27/07/2026 14:14 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55349,7 +55386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C679"/>
+  <dimension ref="A1:C680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64156,16 +64193,29 @@
         </is>
       </c>
       <c r="B677" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C677" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="679">
-      <c r="A679" t="inlineStr">
-        <is>
-          <t>Atualizado: 26/07/2026 11:50 | Total dias: 676</t>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="B678" t="n">
+        <v>1</v>
+      </c>
+      <c r="C678" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Atualizado: 27/07/2026 14:14 | Total dias: 677</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-28 16:30 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2407,6 +2407,43 @@
         </is>
       </c>
       <c r="G53" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>28/07/2026 13:25</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>6217</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -3044,7 +3081,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -5029,7 +5066,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -27067,7 +27104,7 @@
       </c>
       <c r="F471" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G471" t="inlineStr">
@@ -28736,7 +28773,7 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>135</t>
         </is>
       </c>
       <c r="G503" t="inlineStr">
@@ -30148,7 +30185,7 @@
       </c>
       <c r="F530" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G530" t="inlineStr">
@@ -31089,7 +31126,7 @@
       </c>
       <c r="F548" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G548" t="inlineStr">
@@ -33694,7 +33731,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">
@@ -35991,7 +36028,7 @@
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G642" t="inlineStr">
@@ -36695,7 +36732,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 27/07/2026 14:14 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 28/07/2026 13:25 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55371,7 +55408,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 27/07/2026 14:14 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 28/07/2026 13:25 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55386,7 +55423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C680"/>
+  <dimension ref="A1:C681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64206,16 +64243,29 @@
         </is>
       </c>
       <c r="B678" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C678" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="680">
-      <c r="A680" t="inlineStr">
-        <is>
-          <t>Atualizado: 27/07/2026 14:14 | Total dias: 677</t>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="B679" t="n">
+        <v>5</v>
+      </c>
+      <c r="C679" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Atualizado: 28/07/2026 13:25 | Total dias: 678</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-29 16:08 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2444,6 +2444,43 @@
         </is>
       </c>
       <c r="G54" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>29/07/2026 13:03</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>6222</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -7272,7 +7309,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -12774,7 +12811,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -16812,7 +16849,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -33367,7 +33404,7 @@
       </c>
       <c r="F591" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G591" t="inlineStr">
@@ -36732,7 +36769,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 28/07/2026 13:25 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 29/07/2026 13:03 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55408,7 +55445,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 28/07/2026 13:25 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 29/07/2026 13:03 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55423,7 +55460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C681"/>
+  <dimension ref="A1:C682"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64256,16 +64293,29 @@
         </is>
       </c>
       <c r="B679" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C679" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="681">
-      <c r="A681" t="inlineStr">
-        <is>
-          <t>Atualizado: 28/07/2026 13:25 | Total dias: 678</t>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="B680" t="n">
+        <v>2</v>
+      </c>
+      <c r="C680" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Atualizado: 29/07/2026 13:03 | Total dias: 679</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-30 16:11 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2481,6 +2481,43 @@
         </is>
       </c>
       <c r="G55" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>30/07/2026 13:07</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>6226</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -22180,7 +22217,7 @@
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
@@ -23172,7 +23209,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -36769,7 +36806,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 29/07/2026 13:03 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 30/07/2026 13:07 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55445,7 +55482,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 29/07/2026 13:03 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 30/07/2026 13:07 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55460,7 +55497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C682"/>
+  <dimension ref="A1:C683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64306,16 +64343,29 @@
         </is>
       </c>
       <c r="B680" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C680" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="682">
-      <c r="A682" t="inlineStr">
-        <is>
-          <t>Atualizado: 29/07/2026 13:03 | Total dias: 679</t>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="B681" t="n">
+        <v>2</v>
+      </c>
+      <c r="C681" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Atualizado: 30/07/2026 13:07 | Total dias: 680</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-07-31 16:26 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2518,6 +2518,43 @@
         </is>
       </c>
       <c r="G56" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>31/07/2026 13:23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>6230</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -23887,7 +23924,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -36806,7 +36843,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 30/07/2026 13:07 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 31/07/2026 13:23 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55482,7 +55519,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 30/07/2026 13:07 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 31/07/2026 13:23 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55497,7 +55534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C683"/>
+  <dimension ref="A1:C684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64356,16 +64393,29 @@
         </is>
       </c>
       <c r="B681" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C681" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="683">
-      <c r="A683" t="inlineStr">
-        <is>
-          <t>Atualizado: 30/07/2026 13:07 | Total dias: 680</t>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="B682" t="n">
+        <v>3</v>
+      </c>
+      <c r="C682" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Atualizado: 31/07/2026 13:23 | Total dias: 681</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-01 14:46 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2555,6 +2555,43 @@
         </is>
       </c>
       <c r="G57" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>01/08/2026 11:44</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>6232</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -9746,7 +9783,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -16975,7 +17012,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
@@ -36843,7 +36880,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 31/07/2026 13:23 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 01/08/2026 11:44 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55519,7 +55556,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 31/07/2026 13:23 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 01/08/2026 11:44 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55534,7 +55571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C684"/>
+  <dimension ref="A1:C685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64412,10 +64449,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="684">
-      <c r="A684" t="inlineStr">
-        <is>
-          <t>Atualizado: 31/07/2026 13:23 | Total dias: 681</t>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="B683" t="n">
+        <v>2</v>
+      </c>
+      <c r="C683" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Atualizado: 01/08/2026 11:44 | Total dias: 682</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-02 11:14 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2592,6 +2592,43 @@
         </is>
       </c>
       <c r="G58" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>02/08/2026 08:12</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>6238</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -8941,7 +8978,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -9417,7 +9454,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>221</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -11775,7 +11812,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -22239,7 +22276,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>79</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -36880,7 +36917,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 01/08/2026 11:44 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 02/08/2026 08:12 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55556,7 +55593,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 01/08/2026 11:44 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 02/08/2026 08:12 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -64456,7 +64493,7 @@
         </is>
       </c>
       <c r="B683" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C683" t="n">
         <v>0</v>
@@ -64465,7 +64502,7 @@
     <row r="685">
       <c r="A685" t="inlineStr">
         <is>
-          <t>Atualizado: 01/08/2026 11:44 | Total dias: 682</t>
+          <t>Atualizado: 02/08/2026 08:12 | Total dias: 682</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-03 12:51 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2629,6 +2629,43 @@
         </is>
       </c>
       <c r="G59" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>03/08/2026 09:49</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>6241</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -5199,7 +5236,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -6453,7 +6490,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>374</t>
+          <t>376</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -36917,7 +36954,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 02/08/2026 08:12 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 03/08/2026 09:49 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55593,7 +55630,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 02/08/2026 08:12 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 03/08/2026 09:49 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55608,7 +55645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C685"/>
+  <dimension ref="A1:C686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64499,10 +64536,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="685">
-      <c r="A685" t="inlineStr">
-        <is>
-          <t>Atualizado: 02/08/2026 08:12 | Total dias: 682</t>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
+      <c r="B684" t="n">
+        <v>3</v>
+      </c>
+      <c r="C684" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Atualizado: 03/08/2026 09:49 | Total dias: 683</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-04 12:00 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2666,6 +2666,43 @@
         </is>
       </c>
       <c r="G60" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>04/08/2026 08:57</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>6248</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -7176,7 +7213,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -14363,7 +14400,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -16251,7 +16288,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -36954,7 +36991,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 03/08/2026 09:49 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 04/08/2026 08:57 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55630,7 +55667,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 03/08/2026 09:49 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 04/08/2026 08:57 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55645,7 +55682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C686"/>
+  <dimension ref="A1:C688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64549,10 +64586,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="B685" t="n">
+        <v>5</v>
+      </c>
+      <c r="C685" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="686">
       <c r="A686" t="inlineStr">
         <is>
-          <t>Atualizado: 03/08/2026 09:49 | Total dias: 683</t>
+          <t>04/08/2026</t>
+        </is>
+      </c>
+      <c r="B686" t="n">
+        <v>2</v>
+      </c>
+      <c r="C686" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Atualizado: 04/08/2026 08:57 | Total dias: 685</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-05 11:53 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2703,6 +2703,43 @@
         </is>
       </c>
       <c r="G61" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>05/08/2026 08:51</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>6255</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -8687,7 +8724,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -11573,7 +11610,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -12097,7 +12134,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -18741,7 +18778,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
@@ -26107,7 +26144,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
@@ -36991,7 +37028,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 04/08/2026 08:57 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 05/08/2026 08:51 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55667,7 +55704,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 04/08/2026 08:57 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 05/08/2026 08:51 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55682,7 +55719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C688"/>
+  <dimension ref="A1:C689"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64606,16 +64643,29 @@
         </is>
       </c>
       <c r="B686" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C686" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="688">
-      <c r="A688" t="inlineStr">
-        <is>
-          <t>Atualizado: 04/08/2026 08:57 | Total dias: 685</t>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B687" t="n">
+        <v>2</v>
+      </c>
+      <c r="C687" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Atualizado: 05/08/2026 08:51 | Total dias: 686</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-06 11:58 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2740,6 +2740,43 @@
         </is>
       </c>
       <c r="G62" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>06/08/2026 08:56</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>6266</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
         <is>
           <t>519</t>
         </is>
@@ -5571,7 +5608,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -6564,7 +6601,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>376</t>
+          <t>377</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -9089,7 +9126,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -12134,7 +12171,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -24292,12 +24329,12 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>Com este desconto você tem direito a 20% de desconto nas 3 primeiras consultas.</t>
+          <t>20% desconto em todos os serviços e treinamentos ofertados</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>1252</t>
+          <t>1171</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -24337,19 +24374,19 @@
       </c>
       <c r="J412" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>516</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>20% desconto em todos os serviços e treinamentos ofertados</t>
+          <t>Com este desconto você tem direito a 20% de desconto nas 3 primeiras consultas.</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>1171</t>
+          <t>1252</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -24369,7 +24406,7 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -24389,7 +24426,7 @@
       </c>
       <c r="J413" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>588</t>
         </is>
       </c>
     </row>
@@ -24684,7 +24721,7 @@
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
@@ -34027,7 +34064,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">
@@ -37028,7 +37065,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 05/08/2026 08:51 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 06/08/2026 08:56 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55704,7 +55741,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 05/08/2026 08:51 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 06/08/2026 08:56 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
         </is>
       </c>
     </row>
@@ -55719,7 +55756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C689"/>
+  <dimension ref="A1:C690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64656,16 +64693,29 @@
         </is>
       </c>
       <c r="B687" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C687" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="689">
-      <c r="A689" t="inlineStr">
-        <is>
-          <t>Atualizado: 05/08/2026 08:51 | Total dias: 686</t>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
+      <c r="B688" t="n">
+        <v>5</v>
+      </c>
+      <c r="C688" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Atualizado: 06/08/2026 08:56 | Total dias: 687</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-07 10:44 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2779,6 +2779,43 @@
       <c r="G63" t="inlineStr">
         <is>
           <t>519</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>07/08/2026 07:42</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>6286</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>518</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6323,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -6919,7 +6956,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -8709,7 +8746,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -10548,7 +10585,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -12119,7 +12156,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -14422,7 +14459,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -14996,7 +15033,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -21166,7 +21203,7 @@
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
@@ -22319,7 +22356,7 @@
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
@@ -24250,7 +24287,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>61</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -24513,7 +24550,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -27015,7 +27052,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G463" t="inlineStr">
@@ -27541,7 +27578,7 @@
       </c>
       <c r="F473" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>57</t>
         </is>
       </c>
       <c r="G473" t="inlineStr">
@@ -29575,7 +29612,7 @@
       </c>
       <c r="F512" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="G512" t="inlineStr">
@@ -35056,7 +35093,7 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>208</t>
         </is>
       </c>
       <c r="G617" t="inlineStr">
@@ -37065,7 +37102,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 06/08/2026 08:56 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 07/08/2026 07:42 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -37130,7 +37167,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nao cadastrado</t>
+          <t>Lupo / lupo@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -55741,7 +55778,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 06/08/2026 08:56 | Total: 697 | c/ usuario: 178 | s/ usuario: 519</t>
+          <t>Atualizado: 07/08/2026 07:42 | Total: 697 | c/ usuario: 179 | s/ usuario: 518</t>
         </is>
       </c>
     </row>
@@ -55756,7 +55793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C690"/>
+  <dimension ref="A1:C691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64706,16 +64743,29 @@
         </is>
       </c>
       <c r="B688" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C688" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="690">
-      <c r="A690" t="inlineStr">
-        <is>
-          <t>Atualizado: 06/08/2026 08:56 | Total dias: 687</t>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B689" t="n">
+        <v>2</v>
+      </c>
+      <c r="C689" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Atualizado: 07/08/2026 07:42 | Total dias: 688</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-08 10:25 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2816,6 +2816,43 @@
       <c r="G64" t="inlineStr">
         <is>
           <t>518</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08/08/2026 07:21</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>6294</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>515</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3698,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -12208,7 +12245,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -24287,7 +24324,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -29143,7 +29180,7 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>137</t>
         </is>
       </c>
       <c r="G503" t="inlineStr">
@@ -34257,7 +34294,7 @@
       </c>
       <c r="F601" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>65</t>
         </is>
       </c>
       <c r="G601" t="inlineStr">
@@ -37102,7 +37139,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 07/08/2026 07:42 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 08/08/2026 07:21 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55395,7 +55432,7 @@
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>Nao cadastrado</t>
+          <t>Samuel / kiacaiwsmall@hotmail.com</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
@@ -55686,7 +55723,7 @@
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>Nao cadastrado</t>
+          <t>Marcelo Caldas Ribeiro / magoodobrasil@gmail.com</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
@@ -55733,12 +55770,12 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>CCAA</t>
+          <t>CCAA Tatuapé</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>Nao cadastrado</t>
+          <t>SUELLEN LUPO GARCIA / tatuape.corp@ccaa.com.br</t>
         </is>
       </c>
       <c r="D697" t="inlineStr">
@@ -55778,7 +55815,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 07/08/2026 07:42 | Total: 697 | c/ usuario: 179 | s/ usuario: 518</t>
+          <t>Atualizado: 08/08/2026 07:21 | Total: 697 | c/ usuario: 182 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -55793,7 +55830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C691"/>
+  <dimension ref="A1:C692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64756,16 +64793,29 @@
         </is>
       </c>
       <c r="B689" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C689" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="691">
-      <c r="A691" t="inlineStr">
-        <is>
-          <t>Atualizado: 07/08/2026 07:42 | Total dias: 688</t>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="B690" t="n">
+        <v>1</v>
+      </c>
+      <c r="C690" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Atualizado: 08/08/2026 07:21 | Total dias: 689</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-09 10:26 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2851,6 +2851,43 @@
         </is>
       </c>
       <c r="G65" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>09/08/2026 07:23</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>6309</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -7520,7 +7557,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -8731,7 +8768,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -9676,7 +9713,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>222</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -11617,7 +11654,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>146</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -16384,7 +16421,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -18209,7 +18246,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -20198,7 +20235,7 @@
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
@@ -22498,7 +22535,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -24220,7 +24257,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -27037,7 +27074,7 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G462" t="inlineStr">
@@ -31533,7 +31570,7 @@
       </c>
       <c r="F548" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G548" t="inlineStr">
@@ -35130,7 +35167,7 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>209</t>
         </is>
       </c>
       <c r="G617" t="inlineStr">
@@ -35913,7 +35950,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G632" t="inlineStr">
@@ -37139,7 +37176,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 08/08/2026 07:21 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 09/08/2026 07:23 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55815,7 +55852,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 08/08/2026 07:21 | Total: 697 | c/ usuario: 182 | s/ usuario: 515</t>
+          <t>Atualizado: 09/08/2026 07:23 | Total: 697 | c/ usuario: 182 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -55830,7 +55867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C692"/>
+  <dimension ref="A1:C693"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64806,16 +64843,29 @@
         </is>
       </c>
       <c r="B690" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C690" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="692">
-      <c r="A692" t="inlineStr">
-        <is>
-          <t>Atualizado: 08/08/2026 07:21 | Total dias: 689</t>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>09/08/2026</t>
+        </is>
+      </c>
+      <c r="B691" t="n">
+        <v>2</v>
+      </c>
+      <c r="C691" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Atualizado: 09/08/2026 07:23 | Total dias: 690</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-10 11:02 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2888,6 +2888,43 @@
         </is>
       </c>
       <c r="G66" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>10/08/2026 07:59</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>835</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>6314</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -8872,7 +8909,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>144</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -20129,7 +20166,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -29686,7 +29723,7 @@
       </c>
       <c r="F512" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G512" t="inlineStr">
@@ -37176,7 +37213,7 @@
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Atualizado: 09/08/2026 07:23 | Ativas: 835 | Inativas: 0</t>
+          <t>Atualizado: 10/08/2026 07:59 | Ativas: 835 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -55852,7 +55889,7 @@
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 09/08/2026 07:23 | Total: 697 | c/ usuario: 182 | s/ usuario: 515</t>
+          <t>Atualizado: 10/08/2026 07:59 | Total: 697 | c/ usuario: 182 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -55867,7 +55904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C693"/>
+  <dimension ref="A1:C694"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64856,16 +64893,29 @@
         </is>
       </c>
       <c r="B691" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C691" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="693">
-      <c r="A693" t="inlineStr">
-        <is>
-          <t>Atualizado: 09/08/2026 07:23 | Total dias: 690</t>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B692" t="n">
+        <v>1</v>
+      </c>
+      <c r="C692" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Atualizado: 10/08/2026 07:59 | Total dias: 691</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-11 10:47 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2927,6 +2927,43 @@
       <c r="G67" t="inlineStr">
         <is>
           <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>11/08/2026 07:43</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>837</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>6327</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>699</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>516</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J657"/>
+  <dimension ref="A1:J658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -4452,7 +4489,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5547,7 +5584,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>68</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -22572,7 +22609,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>81</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -24398,7 +24435,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>63</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -26277,7 +26314,7 @@
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
@@ -26434,7 +26471,7 @@
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G449" t="inlineStr">
@@ -28836,7 +28873,7 @@
       </c>
       <c r="F495" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G495" t="inlineStr">
@@ -33563,17 +33600,17 @@
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Mais de R$ 350 reais em beneficios exclusivos</t>
         </is>
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>1068</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 350.00</t>
         </is>
       </c>
       <c r="D586" t="inlineStr">
@@ -33588,7 +33625,7 @@
       </c>
       <c r="F586" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G586" t="inlineStr">
@@ -33608,24 +33645,24 @@
       </c>
       <c r="J586" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>957</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 12% de desconto em cirurgias</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>1256</t>
+          <t>1068</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>12.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D587" t="inlineStr">
@@ -33640,7 +33677,7 @@
       </c>
       <c r="F587" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G587" t="inlineStr">
@@ -33660,24 +33697,24 @@
       </c>
       <c r="J587" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>430</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
         <is>
-          <t>Com este voucher você garante 10% de desconto em todos os produtos da loja.</t>
+          <t>Com este cupom você tem direito a 12% de desconto em cirurgias</t>
         </is>
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>1164</t>
+          <t>1256</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>12.00%</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
@@ -33712,24 +33749,24 @@
       </c>
       <c r="J588" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>590</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
         <is>
-          <t>Desconto de 20% em todos os tratamentos corporais e faciais não invasivos! Desconto não é válido para pacotes promocionais.</t>
+          <t>Com este voucher você garante 10% de desconto em todos os produtos da loja.</t>
         </is>
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>1298</t>
+          <t>1164</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D589" t="inlineStr">
@@ -33764,24 +33801,24 @@
       </c>
       <c r="J589" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>510</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
         <is>
-          <t>5 marmitas + 5 sopas por apenas R$ 125,00</t>
+          <t>Desconto de 20% em todos os tratamentos corporais e faciais não invasivos! Desconto não é válido para pacotes promocionais.</t>
         </is>
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1298</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D590" t="inlineStr">
@@ -33816,24 +33853,24 @@
       </c>
       <c r="J590" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>640</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
         <is>
-          <t>15% de descnto em produtos da loja.</t>
+          <t>5 marmitas + 5 sopas por apenas R$ 125,00</t>
         </is>
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>1335</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D591" t="inlineStr">
@@ -33848,7 +33885,7 @@
       </c>
       <c r="F591" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G591" t="inlineStr">
@@ -33868,24 +33905,24 @@
       </c>
       <c r="J591" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>342</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto nos serviços de barba e cabelo.</t>
+          <t>15% de descnto em produtos da loja.</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>1245</t>
+          <t>1335</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D592" t="inlineStr">
@@ -33900,7 +33937,7 @@
       </c>
       <c r="F592" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G592" t="inlineStr">
@@ -33920,24 +33957,24 @@
       </c>
       <c r="J592" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>701</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>Com este cupom você tem direito a 20% de desconto nos serviços de barba e cabelo.</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>1443</t>
+          <t>1245</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D593" t="inlineStr">
@@ -33952,7 +33989,7 @@
       </c>
       <c r="F593" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G593" t="inlineStr">
@@ -33972,19 +34009,19 @@
       </c>
       <c r="J593" t="inlineStr">
         <is>
-          <t>815</t>
+          <t>581</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto para compras feitas através do nosso site.</t>
+          <t>10%OFF</t>
         </is>
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>1443</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
@@ -34024,24 +34061,24 @@
       </c>
       <c r="J594" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>815</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto para Kit Capa e película.</t>
+          <t>Com este cupom você tem direito a 10% de desconto para compras feitas através do nosso site.</t>
         </is>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>1305</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D595" t="inlineStr">
@@ -34076,24 +34113,24 @@
       </c>
       <c r="J595" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>556</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Com este cupom você tem direito a 20% de desconto para Kit Capa e película.</t>
         </is>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1305</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D596" t="inlineStr">
@@ -34103,7 +34140,7 @@
       </c>
       <c r="E596" t="inlineStr">
         <is>
-          <t>-100</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F596" t="inlineStr">
@@ -34128,24 +34165,24 @@
       </c>
       <c r="J596" t="inlineStr">
         <is>
-          <t>716</t>
+          <t>648</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
         <is>
-          <t>15% OFF CARMEL CUMBUCO</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>1393</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D597" t="inlineStr">
@@ -34155,12 +34192,12 @@
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-100</t>
         </is>
       </c>
       <c r="F597" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G597" t="inlineStr">
@@ -34180,24 +34217,24 @@
       </c>
       <c r="J597" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>716</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>10% Off no site</t>
+          <t>15% OFF CARMEL CUMBUCO</t>
         </is>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>1568</t>
+          <t>1393</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D598" t="inlineStr">
@@ -34212,7 +34249,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">
@@ -34232,24 +34269,24 @@
       </c>
       <c r="J598" t="inlineStr">
         <is>
-          <t>927</t>
+          <t>110</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 50% de desconto em nossa consultoria de imagem</t>
+          <t>10% Off no site</t>
         </is>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>1230</t>
+          <t>1568</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
@@ -34264,7 +34301,7 @@
       </c>
       <c r="F599" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G599" t="inlineStr">
@@ -34284,24 +34321,24 @@
       </c>
       <c r="J599" t="inlineStr">
         <is>
-          <t>574</t>
+          <t>927</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>30%OFF</t>
+          <t>Com este cupom você tem direito a 50% de desconto em nossa consultoria de imagem</t>
         </is>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>1446</t>
+          <t>1230</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
@@ -34316,7 +34353,7 @@
       </c>
       <c r="F600" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G600" t="inlineStr">
@@ -34336,24 +34373,24 @@
       </c>
       <c r="J600" t="inlineStr">
         <is>
-          <t>817</t>
+          <t>574</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
         <is>
-          <t>15%OFF</t>
+          <t>30%OFF</t>
         </is>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>1423</t>
+          <t>1446</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D601" t="inlineStr">
@@ -34368,12 +34405,12 @@
       </c>
       <c r="F601" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G601" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H601" t="inlineStr">
@@ -34388,24 +34425,24 @@
       </c>
       <c r="J601" t="inlineStr">
         <is>
-          <t>796</t>
+          <t>817</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto no seu Óculos Sport.</t>
+          <t>15%OFF</t>
         </is>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>1294</t>
+          <t>1423</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D602" t="inlineStr">
@@ -34420,12 +34457,12 @@
       </c>
       <c r="F602" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>65</t>
         </is>
       </c>
       <c r="G602" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H602" t="inlineStr">
@@ -34440,24 +34477,24 @@
       </c>
       <c r="J602" t="inlineStr">
         <is>
-          <t>637</t>
+          <t>796</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>15% OFF</t>
+          <t>Com este cupom você tem direito a 20% de desconto no seu Óculos Sport.</t>
         </is>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>1375</t>
+          <t>1294</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D603" t="inlineStr">
@@ -34472,7 +34509,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G603" t="inlineStr">
@@ -34492,24 +34529,24 @@
       </c>
       <c r="J603" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>637</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
+          <t>15% OFF</t>
         </is>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>1375</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D604" t="inlineStr">
@@ -34524,7 +34561,7 @@
       </c>
       <c r="F604" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G604" t="inlineStr">
@@ -34544,129 +34581,129 @@
       </c>
       <c r="J604" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>750</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
+          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>1114</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 10% de desconto em manutenção e reparos (trocar de telas,baterias,etc)
 Obs: Preços diferenciados para aquisição de aparelhos,air tags,alexa,etc..</t>
         </is>
       </c>
-      <c r="B605" t="inlineStr">
+      <c r="B606" t="inlineStr">
         <is>
           <t>1297</t>
         </is>
       </c>
-      <c r="C605" t="inlineStr">
+      <c r="C606" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D605" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E605" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F605" t="inlineStr">
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G605" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H605" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I605" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J605" t="inlineStr">
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
         <is>
           <t>639</t>
-        </is>
-      </c>
-    </row>
-    <row r="606">
-      <c r="A606" t="inlineStr">
-        <is>
-          <t>VOUCHER DE 200,00</t>
-        </is>
-      </c>
-      <c r="B606" t="inlineStr">
-        <is>
-          <t>1419</t>
-        </is>
-      </c>
-      <c r="C606" t="inlineStr">
-        <is>
-          <t>R$ 200.00</t>
-        </is>
-      </c>
-      <c r="D606" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E606" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F606" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="G606" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H606" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I606" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J606" t="inlineStr">
-        <is>
-          <t>792</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto no seu primeiro pedido.</t>
+          <t>VOUCHER DE 200,00</t>
         </is>
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>1304</t>
+          <t>1419</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 200.00</t>
         </is>
       </c>
       <c r="D607" t="inlineStr">
@@ -34681,7 +34718,7 @@
       </c>
       <c r="F607" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G607" t="inlineStr">
@@ -34701,24 +34738,24 @@
       </c>
       <c r="J607" t="inlineStr">
         <is>
-          <t>646</t>
+          <t>792</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
         <is>
-          <t>4 sessões</t>
+          <t>Com este cupom você tem direito a 10% de desconto no seu primeiro pedido.</t>
         </is>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1304</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
         <is>
-          <t>R$ 500.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D608" t="inlineStr">
@@ -34733,7 +34770,7 @@
       </c>
       <c r="F608" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G608" t="inlineStr">
@@ -34753,24 +34790,24 @@
       </c>
       <c r="J608" t="inlineStr">
         <is>
-          <t>943</t>
+          <t>646</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em todo o nosso cardápio.</t>
+          <t>4 sessões</t>
         </is>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>1241</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 500.00</t>
         </is>
       </c>
       <c r="D609" t="inlineStr">
@@ -34785,7 +34822,7 @@
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G609" t="inlineStr">
@@ -34805,19 +34842,19 @@
       </c>
       <c r="J609" t="inlineStr">
         <is>
-          <t>579</t>
+          <t>943</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto no nosso COMBO de 10 refeições!</t>
+          <t>Com este cupom você tem direito a 10% de desconto em todo o nosso cardápio.</t>
         </is>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>1103</t>
+          <t>1241</t>
         </is>
       </c>
       <c r="C610" t="inlineStr">
@@ -34837,7 +34874,7 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G610" t="inlineStr">
@@ -34857,19 +34894,19 @@
       </c>
       <c r="J610" t="inlineStr">
         <is>
-          <t>453</t>
+          <t>579</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto em nossa loja.</t>
+          <t>Garanta agora 10% de desconto no nosso COMBO de 10 refeições!</t>
         </is>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>1302</t>
+          <t>1103</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
@@ -34889,7 +34926,7 @@
       </c>
       <c r="F611" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G611" t="inlineStr">
@@ -34909,287 +34946,287 @@
       </c>
       <c r="J611" t="inlineStr">
         <is>
-          <t>644</t>
+          <t>453</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
+          <t>Garanta agora 10% de desconto em nossa loja.</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>1302</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>644</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 10% de desconto no seu Óculo de Grau.
 Obs: Válido para primeira compra</t>
         </is>
       </c>
-      <c r="B612" t="inlineStr">
+      <c r="B613" t="inlineStr">
         <is>
           <t>1293</t>
         </is>
       </c>
-      <c r="C612" t="inlineStr">
+      <c r="C613" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D612" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E612" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F612" t="inlineStr">
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G612" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H612" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I612" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J612" t="inlineStr">
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
         <is>
           <t>637</t>
-        </is>
-      </c>
-    </row>
-    <row r="613">
-      <c r="A613" t="inlineStr">
-        <is>
-          <t>10% Off em serviços de cabelo</t>
-        </is>
-      </c>
-      <c r="B613" t="inlineStr">
-        <is>
-          <t>1577</t>
-        </is>
-      </c>
-      <c r="C613" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D613" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E613" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F613" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G613" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H613" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I613" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J613" t="inlineStr">
-        <is>
-          <t>931</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
         <is>
+          <t>10% Off em serviços de cabelo</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>1577</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>931</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
           <t>Você ganhou uma cortesia de 30 minutos de estúdio para gravar o seu contéudo.
 *Válido um por CPF</t>
         </is>
       </c>
-      <c r="B614" t="inlineStr">
+      <c r="B615" t="inlineStr">
         <is>
           <t>1244</t>
         </is>
       </c>
-      <c r="C614" t="inlineStr">
+      <c r="C615" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D614" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E614" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F614" t="inlineStr">
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G614" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H614" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I614" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J614" t="inlineStr">
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
         <is>
           <t>580</t>
         </is>
       </c>
     </row>
-    <row r="615">
-      <c r="A615" t="inlineStr">
+    <row r="616">
+      <c r="A616" t="inlineStr">
         <is>
           <t>Na primeira compra acima de R$50,00 ganhe 4 trufas língua de gato mil delícias
 *Exclusivo para loja do Shopping Iguatemi*</t>
         </is>
       </c>
-      <c r="B615" t="inlineStr">
+      <c r="B616" t="inlineStr">
         <is>
           <t>975</t>
         </is>
       </c>
-      <c r="C615" t="inlineStr">
+      <c r="C616" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D615" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E615" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F615" t="inlineStr">
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G615" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H615" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I615" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J615" t="inlineStr">
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
         <is>
           <t>326</t>
-        </is>
-      </c>
-    </row>
-    <row r="616">
-      <c r="A616" t="inlineStr">
-        <is>
-          <t>10% OFF</t>
-        </is>
-      </c>
-      <c r="B616" t="inlineStr">
-        <is>
-          <t>1512</t>
-        </is>
-      </c>
-      <c r="C616" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D616" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E616" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F616" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G616" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H616" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I616" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J616" t="inlineStr">
-        <is>
-          <t>878</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
         <is>
-          <t>Clientes novos ganha 1 sessão de massagem relaxante e 3 sessões de depilação nas axilas</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>1013</t>
+          <t>1512</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
@@ -35204,7 +35241,7 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G617" t="inlineStr">
@@ -35224,24 +35261,24 @@
       </c>
       <c r="J617" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>878</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em nossos produtos.</t>
+          <t>Clientes novos ganha 1 sessão de massagem relaxante e 3 sessões de depilação nas axilas</t>
         </is>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>1292</t>
+          <t>1013</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D618" t="inlineStr">
@@ -35256,7 +35293,7 @@
       </c>
       <c r="F618" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>209</t>
         </is>
       </c>
       <c r="G618" t="inlineStr">
@@ -35276,124 +35313,124 @@
       </c>
       <c r="J618" t="inlineStr">
         <is>
-          <t>636</t>
+          <t>353</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto em nossos produtos.</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>1292</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
           <t>Desconto dentro do app da Schon com o nome “Schon Green”
 Baixe o APP SCHON e tenha acesso ao desconto do parceiro.</t>
         </is>
       </c>
-      <c r="B619" t="inlineStr">
+      <c r="B620" t="inlineStr">
         <is>
           <t>1288</t>
         </is>
       </c>
-      <c r="C619" t="inlineStr">
+      <c r="C620" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D619" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E619" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F619" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G619" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H619" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I619" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J619" t="inlineStr">
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
         <is>
           <t>619</t>
-        </is>
-      </c>
-    </row>
-    <row r="620">
-      <c r="A620" t="inlineStr">
-        <is>
-          <t>Com este cupom você tem direito a 10% de desconto em nosso cardápio.</t>
-        </is>
-      </c>
-      <c r="B620" t="inlineStr">
-        <is>
-          <t>1207</t>
-        </is>
-      </c>
-      <c r="C620" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D620" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E620" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F620" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="G620" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H620" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I620" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J620" t="inlineStr">
-        <is>
-          <t>547</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>Com este cupom você tem direito a 10% de desconto em nosso cardápio.</t>
         </is>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>1530</t>
+          <t>1207</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
@@ -35413,7 +35450,7 @@
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G621" t="inlineStr">
@@ -35433,129 +35470,129 @@
       </c>
       <c r="J621" t="inlineStr">
         <is>
-          <t>896</t>
+          <t>547</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
         <is>
+          <t>10% OFF</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>1530</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
           <t>Garanta 15% de desconto no valor do curso.
 *Não incluso a taxa de matrícula e o material.</t>
         </is>
       </c>
-      <c r="B622" t="inlineStr">
+      <c r="B623" t="inlineStr">
         <is>
           <t>1093</t>
         </is>
       </c>
-      <c r="C622" t="inlineStr">
+      <c r="C623" t="inlineStr">
         <is>
           <t>15.00%</t>
         </is>
       </c>
-      <c r="D622" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E622" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F622" t="inlineStr">
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G622" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H622" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I622" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J622" t="inlineStr">
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
         <is>
           <t>447</t>
-        </is>
-      </c>
-    </row>
-    <row r="623">
-      <c r="A623" t="inlineStr">
-        <is>
-          <t>Com este cupom você tem direio a 20% de desconto nas compras acima de R$400,00</t>
-        </is>
-      </c>
-      <c r="B623" t="inlineStr">
-        <is>
-          <t>1076</t>
-        </is>
-      </c>
-      <c r="C623" t="inlineStr">
-        <is>
-          <t>20.00%</t>
-        </is>
-      </c>
-      <c r="D623" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E623" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F623" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G623" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H623" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I623" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J623" t="inlineStr">
-        <is>
-          <t>625</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" t="inlineStr">
         <is>
-          <t>Sessão Integrativa</t>
+          <t>Com este cupom você tem direio a 20% de desconto nas compras acima de R$400,00</t>
         </is>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>1588</t>
+          <t>1076</t>
         </is>
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>R$ 120.00</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D624" t="inlineStr">
@@ -35570,7 +35607,7 @@
       </c>
       <c r="F624" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G624" t="inlineStr">
@@ -35590,24 +35627,24 @@
       </c>
       <c r="J624" t="inlineStr">
         <is>
-          <t>943</t>
+          <t>625</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Sessão Integrativa</t>
         </is>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>979</t>
+          <t>1588</t>
         </is>
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 120.00</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
@@ -35622,7 +35659,7 @@
       </c>
       <c r="F625" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G625" t="inlineStr">
@@ -35642,19 +35679,19 @@
       </c>
       <c r="J625" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>943</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
         <is>
-          <t>10% de desconto na consulta presencial com retorno. 10% de desconto na consulta on-line sem retorno.</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>1180</t>
+          <t>979</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
@@ -35674,7 +35711,7 @@
       </c>
       <c r="F626" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G626" t="inlineStr">
@@ -35694,19 +35731,19 @@
       </c>
       <c r="J626" t="inlineStr">
         <is>
-          <t>524</t>
+          <t>329</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>10% de desconto na consulta presencial com retorno. 10% de desconto na consulta on-line sem retorno.</t>
         </is>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>1418</t>
+          <t>1180</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
@@ -35726,7 +35763,7 @@
       </c>
       <c r="F627" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G627" t="inlineStr">
@@ -35746,129 +35783,129 @@
       </c>
       <c r="J627" t="inlineStr">
         <is>
-          <t>791</t>
+          <t>524</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
+          <t>10%OFF</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>1418</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>791</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
           <t>Assessorias de RH
 Garanta agora 10% de desconto em Presencial ou online</t>
         </is>
       </c>
-      <c r="B628" t="inlineStr">
+      <c r="B629" t="inlineStr">
         <is>
           <t>1318</t>
         </is>
       </c>
-      <c r="C628" t="inlineStr">
+      <c r="C629" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D628" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E628" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F628" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G628" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H628" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I628" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J628" t="inlineStr">
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
         <is>
           <t>656</t>
-        </is>
-      </c>
-    </row>
-    <row r="629">
-      <c r="A629" t="inlineStr">
-        <is>
-          <t>30% de desconto em serviços , alinhamento e balanceamento</t>
-        </is>
-      </c>
-      <c r="B629" t="inlineStr">
-        <is>
-          <t>993</t>
-        </is>
-      </c>
-      <c r="C629" t="inlineStr">
-        <is>
-          <t>30.00%</t>
-        </is>
-      </c>
-      <c r="D629" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E629" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F629" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G629" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H629" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I629" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J629" t="inlineStr">
-        <is>
-          <t>338</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>30% de desconto em serviços , alinhamento e balanceamento</t>
         </is>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>993</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>30.00%</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
@@ -35883,7 +35920,7 @@
       </c>
       <c r="F630" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G630" t="inlineStr">
@@ -35903,19 +35940,19 @@
       </c>
       <c r="J630" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>338</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>1442</t>
+          <t>1410</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
@@ -35935,7 +35972,7 @@
       </c>
       <c r="F631" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G631" t="inlineStr">
@@ -35955,24 +35992,24 @@
       </c>
       <c r="J631" t="inlineStr">
         <is>
-          <t>813</t>
+          <t>781</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>15% OFF</t>
+          <t>10%OFF</t>
         </is>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>1559</t>
+          <t>1442</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
@@ -35987,12 +36024,12 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G632" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H632" t="inlineStr">
@@ -36007,24 +36044,24 @@
       </c>
       <c r="J632" t="inlineStr">
         <is>
-          <t>915</t>
+          <t>813</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nos produtos da nossa loja online.</t>
+          <t>15% OFF</t>
         </is>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>1139</t>
+          <t>1559</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
@@ -36039,12 +36076,12 @@
       </c>
       <c r="F633" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G633" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H633" t="inlineStr">
@@ -36059,24 +36096,24 @@
       </c>
       <c r="J633" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>915</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
         <is>
-          <t>17% de desconto em 2024</t>
+          <t>Com este cupom você tem direito a 10% de desconto nos produtos da nossa loja online.</t>
         </is>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>1327</t>
+          <t>1139</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>17.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D634" t="inlineStr">
@@ -36091,7 +36128,7 @@
       </c>
       <c r="F634" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G634" t="inlineStr">
@@ -36111,24 +36148,24 @@
       </c>
       <c r="J634" t="inlineStr">
         <is>
-          <t>663</t>
+          <t>492</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
         <is>
-          <t>GANHE UM PROCEDIMENTO</t>
+          <t>17% de desconto em 2024</t>
         </is>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>1450</t>
+          <t>1327</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17.00%</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
@@ -36143,7 +36180,7 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G635" t="inlineStr">
@@ -36158,187 +36195,187 @@
       </c>
       <c r="I635" t="inlineStr">
         <is>
-          <t>2025-06-01</t>
+          <t>Sem expiracao</t>
         </is>
       </c>
       <c r="J635" t="inlineStr">
         <is>
-          <t>806</t>
+          <t>663</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
+          <t>GANHE UM PROCEDIMENTO</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>806</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 20% de desconto em todos os serviços.
 Trabalhamos com contrato de manutenção e serviços avulsos.</t>
         </is>
       </c>
-      <c r="B636" t="inlineStr">
+      <c r="B637" t="inlineStr">
         <is>
           <t>1225</t>
         </is>
       </c>
-      <c r="C636" t="inlineStr">
+      <c r="C637" t="inlineStr">
         <is>
           <t>20.00%</t>
         </is>
       </c>
-      <c r="D636" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E636" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F636" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G636" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H636" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I636" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J636" t="inlineStr">
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
         <is>
           <t>566</t>
         </is>
       </c>
     </row>
-    <row r="637">
-      <c r="A637" t="inlineStr">
+    <row r="638">
+      <c r="A638" t="inlineStr">
         <is>
           <t>Com este cupom você tem direito a 6% de descontos em nossas peças!
 Obs: Válido para pagamento no crédito.</t>
         </is>
       </c>
-      <c r="B637" t="inlineStr">
+      <c r="B638" t="inlineStr">
         <is>
           <t>1223</t>
         </is>
       </c>
-      <c r="C637" t="inlineStr">
+      <c r="C638" t="inlineStr">
         <is>
           <t>6.00%</t>
         </is>
       </c>
-      <c r="D637" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E637" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F637" t="inlineStr">
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G637" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H637" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I637" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J637" t="inlineStr">
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
         <is>
           <t>563</t>
-        </is>
-      </c>
-    </row>
-    <row r="638">
-      <c r="A638" t="inlineStr">
-        <is>
-          <t>15% de desconto</t>
-        </is>
-      </c>
-      <c r="B638" t="inlineStr">
-        <is>
-          <t>1072</t>
-        </is>
-      </c>
-      <c r="C638" t="inlineStr">
-        <is>
-          <t>15.00%</t>
-        </is>
-      </c>
-      <c r="D638" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F638" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G638" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H638" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I638" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J638" t="inlineStr">
-        <is>
-          <t>434</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>15% de desconto</t>
         </is>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>1586</t>
+          <t>1072</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
@@ -36373,19 +36410,19 @@
       </c>
       <c r="J639" t="inlineStr">
         <is>
-          <t>941</t>
+          <t>434</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nas suas tatoos.</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>1080</t>
+          <t>1586</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
@@ -36405,7 +36442,7 @@
       </c>
       <c r="F640" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G640" t="inlineStr">
@@ -36425,19 +36462,19 @@
       </c>
       <c r="J640" t="inlineStr">
         <is>
-          <t>630</t>
+          <t>941</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>10% Off</t>
+          <t>Com este cupom você tem direito a 10% de desconto nas suas tatoos.</t>
         </is>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>1342</t>
+          <t>1080</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -36457,7 +36494,7 @@
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G641" t="inlineStr">
@@ -36477,19 +36514,19 @@
       </c>
       <c r="J641" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>630</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>10% Off</t>
         </is>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>1498</t>
+          <t>1342</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -36509,7 +36546,7 @@
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G642" t="inlineStr">
@@ -36529,24 +36566,24 @@
       </c>
       <c r="J642" t="inlineStr">
         <is>
-          <t>871</t>
+          <t>714</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>Frete grátis nas compras acima de 50 reais.</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>1055</t>
+          <t>1498</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D643" t="inlineStr">
@@ -36561,7 +36598,7 @@
       </c>
       <c r="F643" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G643" t="inlineStr">
@@ -36581,24 +36618,24 @@
       </c>
       <c r="J643" t="inlineStr">
         <is>
-          <t>418</t>
+          <t>871</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>Frete grátis nas compras acima de 50 reais.</t>
         </is>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>1539</t>
+          <t>1055</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
@@ -36633,19 +36670,19 @@
       </c>
       <c r="J644" t="inlineStr">
         <is>
-          <t>906</t>
+          <t>418</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>1355</t>
+          <t>1539</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -36665,7 +36702,7 @@
       </c>
       <c r="F645" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G645" t="inlineStr">
@@ -36685,24 +36722,24 @@
       </c>
       <c r="J645" t="inlineStr">
         <is>
-          <t>737</t>
+          <t>906</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
         <is>
-          <t>15% de desconto ( não válido às sextas e sábados)</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>1026</t>
+          <t>1355</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
@@ -36717,7 +36754,7 @@
       </c>
       <c r="F646" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G646" t="inlineStr">
@@ -36737,19 +36774,19 @@
       </c>
       <c r="J646" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>737</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
         <is>
-          <t>15% de desconto nos serviços de cílios e design de sobrancelhas</t>
+          <t>15% de desconto ( não válido às sextas e sábados)</t>
         </is>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>1026</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -36769,7 +36806,7 @@
       </c>
       <c r="F647" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G647" t="inlineStr">
@@ -36789,24 +36826,24 @@
       </c>
       <c r="J647" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>361</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
         <is>
-          <t>A cada 1 real gasto na loja é convertido em ponto e o aluno poderá acumular ou usar de imediato.</t>
+          <t>15% de desconto nos serviços de cílios e design de sobrancelhas</t>
         </is>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>1188</t>
+          <t>995</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D648" t="inlineStr">
@@ -36841,24 +36878,24 @@
       </c>
       <c r="J648" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>340</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>A cada 1 real gasto na loja é convertido em ponto e o aluno poderá acumular ou usar de imediato.</t>
         </is>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>1515</t>
+          <t>1188</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D649" t="inlineStr">
@@ -36893,24 +36930,24 @@
       </c>
       <c r="J649" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>532</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t>Avaliação Facial Personalizada com IA</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1515</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
@@ -36925,7 +36962,7 @@
       </c>
       <c r="F650" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G650" t="inlineStr">
@@ -36945,124 +36982,124 @@
       </c>
       <c r="J650" t="inlineStr">
         <is>
-          <t>873</t>
+          <t>881</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
+          <t>Avaliação Facial Personalizada com IA</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>873</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
           <t>15% de desconto (não é válido para joias em promoção, alianças, relógios e best seller)
 Válido apenas na loja do Riomar Papicu.</t>
         </is>
       </c>
-      <c r="B651" t="inlineStr">
+      <c r="B652" t="inlineStr">
         <is>
           <t>1320</t>
         </is>
       </c>
-      <c r="C651" t="inlineStr">
+      <c r="C652" t="inlineStr">
         <is>
           <t>15.00%</t>
         </is>
       </c>
-      <c r="D651" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E651" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F651" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G651" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H651" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I651" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J651" t="inlineStr">
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
         <is>
           <t>657</t>
-        </is>
-      </c>
-    </row>
-    <row r="652">
-      <c r="A652" t="inlineStr">
-        <is>
-          <t>10% de desconto em todos os produtos da loja. Válido apenas para pagamentos por cartão de credito.</t>
-        </is>
-      </c>
-      <c r="B652" t="inlineStr">
-        <is>
-          <t>1191</t>
-        </is>
-      </c>
-      <c r="C652" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D652" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E652" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F652" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G652" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H652" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I652" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J652" t="inlineStr">
-        <is>
-          <t>533</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>10% de desconto em qualquer produto (lentes e armações)</t>
+          <t>10% de desconto em todos os produtos da loja. Válido apenas para pagamentos por cartão de credito.</t>
         </is>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>1014</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
@@ -37102,19 +37139,19 @@
       </c>
       <c r="J653" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>533</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nas suas compras.</t>
+          <t>10% de desconto em qualquer produto (lentes e armações)</t>
         </is>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>1131</t>
+          <t>1014</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
@@ -37154,66 +37191,118 @@
       </c>
       <c r="J654" t="inlineStr">
         <is>
-          <t>484</t>
+          <t>354</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto nas suas compras.</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>1131</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>484</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 20% de desconto nas compras em nossa loja.</t>
         </is>
       </c>
-      <c r="B655" t="inlineStr">
+      <c r="B656" t="inlineStr">
         <is>
           <t>1125</t>
         </is>
       </c>
-      <c r="C655" t="inlineStr">
+      <c r="C656" t="inlineStr">
         <is>
           <t>20.00%</t>
         </is>
       </c>
-      <c r="D655" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E655" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F655" t="inlineStr">
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G655" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H655" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I655" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J655" t="inlineStr">
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
         <is>
           <t>478</t>
         </is>
       </c>
     </row>
-    <row r="657">
-      <c r="A657" t="inlineStr">
-        <is>
-          <t>Atualizado: 10/08/2026 07:59 | Ativas: 835 | Inativas: 0</t>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Atualizado: 11/08/2026 07:43 | Ativas: 837 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -37228,7 +37317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E700"/>
+  <dimension ref="A1:E702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55886,10 +55975,64 @@
         <v>18</v>
       </c>
     </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>957</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Atlas Quiropraxia</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Tiago Rodrigues / contato@atlasquiropraxia.com.br</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>SAÚDE E BEM ESTAR</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
     <row r="700">
       <c r="A700" t="inlineStr">
         <is>
-          <t>Atualizado: 10/08/2026 07:59 | Total: 697 | c/ usuario: 182 | s/ usuario: 515</t>
+          <t>958</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Especiarias Aromas Ltda</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Nao cadastrado</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>DIVERSOS</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>Atualizado: 11/08/2026 07:43 | Total: 699 | c/ usuario: 183 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -55904,7 +56047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C694"/>
+  <dimension ref="A1:C695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64883,7 +65026,7 @@
         <v>14</v>
       </c>
       <c r="C690" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="691">
@@ -64906,16 +65049,29 @@
         </is>
       </c>
       <c r="B692" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C692" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="694">
-      <c r="A694" t="inlineStr">
-        <is>
-          <t>Atualizado: 10/08/2026 07:59 | Total dias: 691</t>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="B693" t="n">
+        <v>3</v>
+      </c>
+      <c r="C693" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Atualizado: 11/08/2026 07:43 | Total dias: 692</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-13 10:54 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -2999,6 +2999,43 @@
         </is>
       </c>
       <c r="G69" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>13/08/2026 07:51</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>839</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>6353</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -16271,7 +16308,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -28389,7 +28426,7 @@
       </c>
       <c r="F485" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G485" t="inlineStr">
@@ -29380,7 +29417,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>138</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -32305,7 +32342,7 @@
       </c>
       <c r="F560" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G560" t="inlineStr">
@@ -35330,7 +35367,7 @@
       </c>
       <c r="F618" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G618" t="inlineStr">
@@ -35382,7 +35419,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>213</t>
         </is>
       </c>
       <c r="G619" t="inlineStr">
@@ -37443,7 +37480,7 @@
     <row r="660">
       <c r="A660" t="inlineStr">
         <is>
-          <t>Atualizado: 12/08/2026 07:51 | Ativas: 839 | Inativas: 0</t>
+          <t>Atualizado: 13/08/2026 07:51 | Ativas: 839 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56227,7 +56264,7 @@
     <row r="704">
       <c r="A704" t="inlineStr">
         <is>
-          <t>Atualizado: 12/08/2026 07:51 | Total: 701 | c/ usuario: 186 | s/ usuario: 515</t>
+          <t>Atualizado: 13/08/2026 07:51 | Total: 701 | c/ usuario: 186 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -56242,7 +56279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C696"/>
+  <dimension ref="A1:C697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65270,16 +65307,29 @@
         </is>
       </c>
       <c r="B694" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C694" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="696">
-      <c r="A696" t="inlineStr">
-        <is>
-          <t>Atualizado: 12/08/2026 07:51 | Total dias: 693</t>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>13/08/2026</t>
+        </is>
+      </c>
+      <c r="B695" t="n">
+        <v>5</v>
+      </c>
+      <c r="C695" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Atualizado: 13/08/2026 07:51 | Total dias: 694</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-14 10:49 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3036,6 +3036,43 @@
         </is>
       </c>
       <c r="G70" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>14/08/2026 07:46</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>839</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>6364</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -3673,7 +3710,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -5658,7 +5695,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -11802,7 +11839,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -15307,7 +15344,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -26440,7 +26477,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
@@ -27537,7 +27574,7 @@
       </c>
       <c r="F468" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G468" t="inlineStr">
@@ -34739,7 +34776,7 @@
       </c>
       <c r="F606" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G606" t="inlineStr">
@@ -37480,7 +37517,7 @@
     <row r="660">
       <c r="A660" t="inlineStr">
         <is>
-          <t>Atualizado: 13/08/2026 07:51 | Ativas: 839 | Inativas: 0</t>
+          <t>Atualizado: 14/08/2026 07:46 | Ativas: 839 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56264,7 +56301,7 @@
     <row r="704">
       <c r="A704" t="inlineStr">
         <is>
-          <t>Atualizado: 13/08/2026 07:51 | Total: 701 | c/ usuario: 186 | s/ usuario: 515</t>
+          <t>Atualizado: 14/08/2026 07:46 | Total: 701 | c/ usuario: 186 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -56279,7 +56316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C697"/>
+  <dimension ref="A1:C698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65320,16 +65357,29 @@
         </is>
       </c>
       <c r="B695" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C695" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="697">
-      <c r="A697" t="inlineStr">
-        <is>
-          <t>Atualizado: 13/08/2026 07:51 | Total dias: 694</t>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
+      <c r="B696" t="n">
+        <v>1</v>
+      </c>
+      <c r="C696" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Atualizado: 14/08/2026 07:46 | Total dias: 695</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-15 10:15 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3075,6 +3075,43 @@
       <c r="G71" t="inlineStr">
         <is>
           <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>15/08/2026 07:12</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>840</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>6378</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>702</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>516</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J660"/>
+  <dimension ref="A1:J661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -3920,7 +3957,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -7953,7 +7990,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -24442,7 +24479,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -29454,7 +29491,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>139</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -31597,7 +31634,7 @@
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G545" t="inlineStr">
@@ -32223,7 +32260,7 @@
       </c>
       <c r="F557" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G557" t="inlineStr">
@@ -33606,17 +33643,17 @@
     <row r="584">
       <c r="A584" t="inlineStr">
         <is>
-          <t>15% de desconto nos serviços de cílios</t>
+          <t>20% OFF</t>
         </is>
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>997</t>
+          <t>1609</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D584" t="inlineStr">
@@ -33626,7 +33663,7 @@
       </c>
       <c r="E584" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="F584" t="inlineStr">
@@ -33651,24 +33688,24 @@
       </c>
       <c r="J584" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>961</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em SIPAT para Empresas.</t>
+          <t>15% de desconto nos serviços de cílios</t>
         </is>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>997</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D585" t="inlineStr">
@@ -33683,7 +33720,7 @@
       </c>
       <c r="F585" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G585" t="inlineStr">
@@ -33703,129 +33740,129 @@
       </c>
       <c r="J585" t="inlineStr">
         <is>
-          <t>608</t>
+          <t>341</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto em SIPAT para Empresas.</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>1280</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>608</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
           <t>10% em qualquer serviço 
 *Atendemos em domicilio!*</t>
         </is>
       </c>
-      <c r="B586" t="inlineStr">
+      <c r="B587" t="inlineStr">
         <is>
           <t>1029</t>
         </is>
       </c>
-      <c r="C586" t="inlineStr">
+      <c r="C587" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D586" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E586" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F586" t="inlineStr">
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G586" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H586" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I586" t="inlineStr">
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J586" t="inlineStr">
+      <c r="J587" t="inlineStr">
         <is>
           <t>364</t>
-        </is>
-      </c>
-    </row>
-    <row r="587">
-      <c r="A587" t="inlineStr">
-        <is>
-          <t>Mais de R$ 350 reais em beneficios exclusivos</t>
-        </is>
-      </c>
-      <c r="B587" t="inlineStr">
-        <is>
-          <t>1605</t>
-        </is>
-      </c>
-      <c r="C587" t="inlineStr">
-        <is>
-          <t>R$ 350.00</t>
-        </is>
-      </c>
-      <c r="D587" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E587" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F587" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G587" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H587" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I587" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J587" t="inlineStr">
-        <is>
-          <t>957</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Mais de R$ 350 reais em beneficios exclusivos</t>
         </is>
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>1068</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 350.00</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
@@ -33840,7 +33877,7 @@
       </c>
       <c r="F588" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G588" t="inlineStr">
@@ -33860,24 +33897,24 @@
       </c>
       <c r="J588" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>957</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 12% de desconto em cirurgias</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>1256</t>
+          <t>1068</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>12.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D589" t="inlineStr">
@@ -33892,7 +33929,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G589" t="inlineStr">
@@ -33912,24 +33949,24 @@
       </c>
       <c r="J589" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>430</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
         <is>
-          <t>Com este voucher você garante 10% de desconto em todos os produtos da loja.</t>
+          <t>Com este cupom você tem direito a 12% de desconto em cirurgias</t>
         </is>
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>1164</t>
+          <t>1256</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>12.00%</t>
         </is>
       </c>
       <c r="D590" t="inlineStr">
@@ -33964,24 +34001,24 @@
       </c>
       <c r="J590" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>590</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
         <is>
-          <t>Desconto de 20% em todos os tratamentos corporais e faciais não invasivos! Desconto não é válido para pacotes promocionais.</t>
+          <t>Com este voucher você garante 10% de desconto em todos os produtos da loja.</t>
         </is>
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>1298</t>
+          <t>1164</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D591" t="inlineStr">
@@ -34016,24 +34053,24 @@
       </c>
       <c r="J591" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>510</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
         <is>
-          <t>5 marmitas + 5 sopas por apenas R$ 125,00</t>
+          <t>Desconto de 20% em todos os tratamentos corporais e faciais não invasivos! Desconto não é válido para pacotes promocionais.</t>
         </is>
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1298</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D592" t="inlineStr">
@@ -34068,24 +34105,24 @@
       </c>
       <c r="J592" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>640</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>15% de descnto em produtos da loja.</t>
+          <t>5 marmitas + 5 sopas por apenas R$ 125,00</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>1335</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D593" t="inlineStr">
@@ -34100,7 +34137,7 @@
       </c>
       <c r="F593" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G593" t="inlineStr">
@@ -34120,24 +34157,24 @@
       </c>
       <c r="J593" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>342</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto nos serviços de barba e cabelo.</t>
+          <t>15% de descnto em produtos da loja.</t>
         </is>
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>1245</t>
+          <t>1335</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D594" t="inlineStr">
@@ -34152,7 +34189,7 @@
       </c>
       <c r="F594" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G594" t="inlineStr">
@@ -34172,24 +34209,24 @@
       </c>
       <c r="J594" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>701</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>Com este cupom você tem direito a 20% de desconto nos serviços de barba e cabelo.</t>
         </is>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>1443</t>
+          <t>1245</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D595" t="inlineStr">
@@ -34204,7 +34241,7 @@
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G595" t="inlineStr">
@@ -34224,19 +34261,19 @@
       </c>
       <c r="J595" t="inlineStr">
         <is>
-          <t>815</t>
+          <t>581</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto para compras feitas através do nosso site.</t>
+          <t>10%OFF</t>
         </is>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>1443</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
@@ -34276,24 +34313,24 @@
       </c>
       <c r="J596" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>815</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto para Kit Capa e película.</t>
+          <t>Com este cupom você tem direito a 10% de desconto para compras feitas através do nosso site.</t>
         </is>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>1305</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D597" t="inlineStr">
@@ -34328,24 +34365,24 @@
       </c>
       <c r="J597" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>556</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Com este cupom você tem direito a 20% de desconto para Kit Capa e película.</t>
         </is>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1305</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D598" t="inlineStr">
@@ -34355,7 +34392,7 @@
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>-100</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F598" t="inlineStr">
@@ -34380,24 +34417,24 @@
       </c>
       <c r="J598" t="inlineStr">
         <is>
-          <t>716</t>
+          <t>648</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>15% OFF CARMEL CUMBUCO</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>1393</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
@@ -34407,12 +34444,12 @@
       </c>
       <c r="E599" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-100</t>
         </is>
       </c>
       <c r="F599" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G599" t="inlineStr">
@@ -34432,24 +34469,24 @@
       </c>
       <c r="J599" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>716</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>10% Off no site</t>
+          <t>15% OFF CARMEL CUMBUCO</t>
         </is>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>1568</t>
+          <t>1393</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
@@ -34464,7 +34501,7 @@
       </c>
       <c r="F600" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G600" t="inlineStr">
@@ -34484,24 +34521,24 @@
       </c>
       <c r="J600" t="inlineStr">
         <is>
-          <t>927</t>
+          <t>110</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 50% de desconto em nossa consultoria de imagem</t>
+          <t>10% Off no site</t>
         </is>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>1230</t>
+          <t>1568</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D601" t="inlineStr">
@@ -34516,7 +34553,7 @@
       </c>
       <c r="F601" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G601" t="inlineStr">
@@ -34536,24 +34573,24 @@
       </c>
       <c r="J601" t="inlineStr">
         <is>
-          <t>574</t>
+          <t>927</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
         <is>
-          <t>30%OFF</t>
+          <t>Com este cupom você tem direito a 50% de desconto em nossa consultoria de imagem</t>
         </is>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>1446</t>
+          <t>1230</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="D602" t="inlineStr">
@@ -34568,7 +34605,7 @@
       </c>
       <c r="F602" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G602" t="inlineStr">
@@ -34588,24 +34625,24 @@
       </c>
       <c r="J602" t="inlineStr">
         <is>
-          <t>817</t>
+          <t>574</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>15%OFF</t>
+          <t>30%OFF</t>
         </is>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>1423</t>
+          <t>1446</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D603" t="inlineStr">
@@ -34620,12 +34657,12 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G603" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H603" t="inlineStr">
@@ -34640,24 +34677,24 @@
       </c>
       <c r="J603" t="inlineStr">
         <is>
-          <t>796</t>
+          <t>817</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto no seu Óculos Sport.</t>
+          <t>15%OFF</t>
         </is>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>1294</t>
+          <t>1423</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D604" t="inlineStr">
@@ -34672,12 +34709,12 @@
       </c>
       <c r="F604" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G604" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H604" t="inlineStr">
@@ -34692,24 +34729,24 @@
       </c>
       <c r="J604" t="inlineStr">
         <is>
-          <t>637</t>
+          <t>796</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>15% OFF</t>
+          <t>Com este cupom você tem direito a 20% de desconto no seu Óculos Sport.</t>
         </is>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>1375</t>
+          <t>1294</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D605" t="inlineStr">
@@ -34724,7 +34761,7 @@
       </c>
       <c r="F605" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G605" t="inlineStr">
@@ -34744,24 +34781,24 @@
       </c>
       <c r="J605" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>637</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
+          <t>15% OFF</t>
         </is>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>1375</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D606" t="inlineStr">
@@ -34776,7 +34813,7 @@
       </c>
       <c r="F606" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G606" t="inlineStr">
@@ -34796,129 +34833,129 @@
       </c>
       <c r="J606" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>750</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
+          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>1114</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 10% de desconto em manutenção e reparos (trocar de telas,baterias,etc)
 Obs: Preços diferenciados para aquisição de aparelhos,air tags,alexa,etc..</t>
         </is>
       </c>
-      <c r="B607" t="inlineStr">
+      <c r="B608" t="inlineStr">
         <is>
           <t>1297</t>
         </is>
       </c>
-      <c r="C607" t="inlineStr">
+      <c r="C608" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D607" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E607" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F607" t="inlineStr">
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G607" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H607" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I607" t="inlineStr">
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J607" t="inlineStr">
+      <c r="J608" t="inlineStr">
         <is>
           <t>639</t>
-        </is>
-      </c>
-    </row>
-    <row r="608">
-      <c r="A608" t="inlineStr">
-        <is>
-          <t>VOUCHER DE 200,00</t>
-        </is>
-      </c>
-      <c r="B608" t="inlineStr">
-        <is>
-          <t>1419</t>
-        </is>
-      </c>
-      <c r="C608" t="inlineStr">
-        <is>
-          <t>R$ 200.00</t>
-        </is>
-      </c>
-      <c r="D608" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E608" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F608" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="G608" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H608" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I608" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J608" t="inlineStr">
-        <is>
-          <t>792</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto no seu primeiro pedido.</t>
+          <t>VOUCHER DE 200,00</t>
         </is>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>1304</t>
+          <t>1419</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 200.00</t>
         </is>
       </c>
       <c r="D609" t="inlineStr">
@@ -34933,7 +34970,7 @@
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G609" t="inlineStr">
@@ -34953,24 +34990,24 @@
       </c>
       <c r="J609" t="inlineStr">
         <is>
-          <t>646</t>
+          <t>792</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
         <is>
-          <t>4 sessões</t>
+          <t>Com este cupom você tem direito a 10% de desconto no seu primeiro pedido.</t>
         </is>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1304</t>
         </is>
       </c>
       <c r="C610" t="inlineStr">
         <is>
-          <t>R$ 500.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D610" t="inlineStr">
@@ -34985,7 +35022,7 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G610" t="inlineStr">
@@ -35005,24 +35042,24 @@
       </c>
       <c r="J610" t="inlineStr">
         <is>
-          <t>943</t>
+          <t>646</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em todo o nosso cardápio.</t>
+          <t>4 sessões</t>
         </is>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>1241</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 500.00</t>
         </is>
       </c>
       <c r="D611" t="inlineStr">
@@ -35037,7 +35074,7 @@
       </c>
       <c r="F611" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G611" t="inlineStr">
@@ -35057,19 +35094,19 @@
       </c>
       <c r="J611" t="inlineStr">
         <is>
-          <t>579</t>
+          <t>943</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto no nosso COMBO de 10 refeições!</t>
+          <t>Com este cupom você tem direito a 10% de desconto em todo o nosso cardápio.</t>
         </is>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>1103</t>
+          <t>1241</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
@@ -35089,7 +35126,7 @@
       </c>
       <c r="F612" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G612" t="inlineStr">
@@ -35109,19 +35146,19 @@
       </c>
       <c r="J612" t="inlineStr">
         <is>
-          <t>453</t>
+          <t>579</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto em nossa loja.</t>
+          <t>Garanta agora 10% de desconto no nosso COMBO de 10 refeições!</t>
         </is>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>1302</t>
+          <t>1103</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
@@ -35141,7 +35178,7 @@
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G613" t="inlineStr">
@@ -35161,287 +35198,287 @@
       </c>
       <c r="J613" t="inlineStr">
         <is>
-          <t>644</t>
+          <t>453</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
         <is>
+          <t>Garanta agora 10% de desconto em nossa loja.</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>1302</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>644</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 10% de desconto no seu Óculo de Grau.
 Obs: Válido para primeira compra</t>
         </is>
       </c>
-      <c r="B614" t="inlineStr">
+      <c r="B615" t="inlineStr">
         <is>
           <t>1293</t>
         </is>
       </c>
-      <c r="C614" t="inlineStr">
+      <c r="C615" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D614" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E614" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F614" t="inlineStr">
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G614" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H614" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I614" t="inlineStr">
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J614" t="inlineStr">
+      <c r="J615" t="inlineStr">
         <is>
           <t>637</t>
-        </is>
-      </c>
-    </row>
-    <row r="615">
-      <c r="A615" t="inlineStr">
-        <is>
-          <t>10% Off em serviços de cabelo</t>
-        </is>
-      </c>
-      <c r="B615" t="inlineStr">
-        <is>
-          <t>1577</t>
-        </is>
-      </c>
-      <c r="C615" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D615" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E615" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F615" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G615" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H615" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I615" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J615" t="inlineStr">
-        <is>
-          <t>931</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
         <is>
+          <t>10% Off em serviços de cabelo</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>1577</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>931</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
           <t>Você ganhou uma cortesia de 30 minutos de estúdio para gravar o seu contéudo.
 *Válido um por CPF</t>
         </is>
       </c>
-      <c r="B616" t="inlineStr">
+      <c r="B617" t="inlineStr">
         <is>
           <t>1244</t>
         </is>
       </c>
-      <c r="C616" t="inlineStr">
+      <c r="C617" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D616" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E616" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F616" t="inlineStr">
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G616" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H616" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I616" t="inlineStr">
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J616" t="inlineStr">
+      <c r="J617" t="inlineStr">
         <is>
           <t>580</t>
         </is>
       </c>
     </row>
-    <row r="617">
-      <c r="A617" t="inlineStr">
+    <row r="618">
+      <c r="A618" t="inlineStr">
         <is>
           <t>Na primeira compra acima de R$50,00 ganhe 4 trufas língua de gato mil delícias
 *Exclusivo para loja do Shopping Iguatemi*</t>
         </is>
       </c>
-      <c r="B617" t="inlineStr">
+      <c r="B618" t="inlineStr">
         <is>
           <t>975</t>
         </is>
       </c>
-      <c r="C617" t="inlineStr">
+      <c r="C618" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D617" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E617" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F617" t="inlineStr">
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G617" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H617" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I617" t="inlineStr">
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J617" t="inlineStr">
+      <c r="J618" t="inlineStr">
         <is>
           <t>326</t>
-        </is>
-      </c>
-    </row>
-    <row r="618">
-      <c r="A618" t="inlineStr">
-        <is>
-          <t>10% OFF</t>
-        </is>
-      </c>
-      <c r="B618" t="inlineStr">
-        <is>
-          <t>1512</t>
-        </is>
-      </c>
-      <c r="C618" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D618" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E618" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F618" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G618" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H618" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I618" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J618" t="inlineStr">
-        <is>
-          <t>878</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>Clientes novos ganha 1 sessão de massagem relaxante e 3 sessões de depilação nas axilas</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>1013</t>
+          <t>1512</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
@@ -35456,7 +35493,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G619" t="inlineStr">
@@ -35476,24 +35513,24 @@
       </c>
       <c r="J619" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>878</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em nossos produtos.</t>
+          <t>Clientes novos ganha 1 sessão de massagem relaxante e 3 sessões de depilação nas axilas</t>
         </is>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>1292</t>
+          <t>1013</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
@@ -35508,7 +35545,7 @@
       </c>
       <c r="F620" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>214</t>
         </is>
       </c>
       <c r="G620" t="inlineStr">
@@ -35528,124 +35565,124 @@
       </c>
       <c r="J620" t="inlineStr">
         <is>
-          <t>636</t>
+          <t>353</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto em nossos produtos.</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>1292</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
           <t>Desconto dentro do app da Schon com o nome “Schon Green”
 Baixe o APP SCHON e tenha acesso ao desconto do parceiro.</t>
         </is>
       </c>
-      <c r="B621" t="inlineStr">
+      <c r="B622" t="inlineStr">
         <is>
           <t>1288</t>
         </is>
       </c>
-      <c r="C621" t="inlineStr">
+      <c r="C622" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D621" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E621" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F621" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G621" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H621" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I621" t="inlineStr">
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J621" t="inlineStr">
+      <c r="J622" t="inlineStr">
         <is>
           <t>619</t>
-        </is>
-      </c>
-    </row>
-    <row r="622">
-      <c r="A622" t="inlineStr">
-        <is>
-          <t>Com este cupom você tem direito a 10% de desconto em nosso cardápio.</t>
-        </is>
-      </c>
-      <c r="B622" t="inlineStr">
-        <is>
-          <t>1207</t>
-        </is>
-      </c>
-      <c r="C622" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D622" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E622" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F622" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="G622" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H622" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I622" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J622" t="inlineStr">
-        <is>
-          <t>547</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>Com este cupom você tem direito a 10% de desconto em nosso cardápio.</t>
         </is>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>1530</t>
+          <t>1207</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
@@ -35665,7 +35702,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -35685,129 +35722,129 @@
       </c>
       <c r="J623" t="inlineStr">
         <is>
-          <t>896</t>
+          <t>547</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" t="inlineStr">
         <is>
+          <t>10% OFF</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>1530</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
           <t>Garanta 15% de desconto no valor do curso.
 *Não incluso a taxa de matrícula e o material.</t>
         </is>
       </c>
-      <c r="B624" t="inlineStr">
+      <c r="B625" t="inlineStr">
         <is>
           <t>1093</t>
         </is>
       </c>
-      <c r="C624" t="inlineStr">
+      <c r="C625" t="inlineStr">
         <is>
           <t>15.00%</t>
         </is>
       </c>
-      <c r="D624" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E624" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F624" t="inlineStr">
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G624" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H624" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I624" t="inlineStr">
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J624" t="inlineStr">
+      <c r="J625" t="inlineStr">
         <is>
           <t>447</t>
-        </is>
-      </c>
-    </row>
-    <row r="625">
-      <c r="A625" t="inlineStr">
-        <is>
-          <t>Com este cupom você tem direio a 20% de desconto nas compras acima de R$400,00</t>
-        </is>
-      </c>
-      <c r="B625" t="inlineStr">
-        <is>
-          <t>1076</t>
-        </is>
-      </c>
-      <c r="C625" t="inlineStr">
-        <is>
-          <t>20.00%</t>
-        </is>
-      </c>
-      <c r="D625" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E625" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F625" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G625" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H625" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I625" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J625" t="inlineStr">
-        <is>
-          <t>625</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
         <is>
-          <t>Sessão Integrativa</t>
+          <t>Com este cupom você tem direio a 20% de desconto nas compras acima de R$400,00</t>
         </is>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>1588</t>
+          <t>1076</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>R$ 120.00</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
@@ -35822,7 +35859,7 @@
       </c>
       <c r="F626" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G626" t="inlineStr">
@@ -35842,24 +35879,24 @@
       </c>
       <c r="J626" t="inlineStr">
         <is>
-          <t>943</t>
+          <t>625</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Sessão Integrativa</t>
         </is>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>979</t>
+          <t>1588</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 120.00</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
@@ -35874,7 +35911,7 @@
       </c>
       <c r="F627" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G627" t="inlineStr">
@@ -35894,19 +35931,19 @@
       </c>
       <c r="J627" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>943</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>10% de desconto na consulta presencial com retorno. 10% de desconto na consulta on-line sem retorno.</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>1180</t>
+          <t>979</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -35926,7 +35963,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G628" t="inlineStr">
@@ -35946,19 +35983,19 @@
       </c>
       <c r="J628" t="inlineStr">
         <is>
-          <t>524</t>
+          <t>329</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>10% de desconto na consulta presencial com retorno. 10% de desconto na consulta on-line sem retorno.</t>
         </is>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>1418</t>
+          <t>1180</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
@@ -35978,7 +36015,7 @@
       </c>
       <c r="F629" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G629" t="inlineStr">
@@ -35998,129 +36035,129 @@
       </c>
       <c r="J629" t="inlineStr">
         <is>
-          <t>791</t>
+          <t>524</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
+          <t>10%OFF</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>1418</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>791</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
           <t>Assessorias de RH
 Garanta agora 10% de desconto em Presencial ou online</t>
         </is>
       </c>
-      <c r="B630" t="inlineStr">
+      <c r="B631" t="inlineStr">
         <is>
           <t>1318</t>
         </is>
       </c>
-      <c r="C630" t="inlineStr">
+      <c r="C631" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D630" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E630" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F630" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G630" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H630" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I630" t="inlineStr">
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J630" t="inlineStr">
+      <c r="J631" t="inlineStr">
         <is>
           <t>656</t>
-        </is>
-      </c>
-    </row>
-    <row r="631">
-      <c r="A631" t="inlineStr">
-        <is>
-          <t>30% de desconto em serviços , alinhamento e balanceamento</t>
-        </is>
-      </c>
-      <c r="B631" t="inlineStr">
-        <is>
-          <t>993</t>
-        </is>
-      </c>
-      <c r="C631" t="inlineStr">
-        <is>
-          <t>30.00%</t>
-        </is>
-      </c>
-      <c r="D631" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E631" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F631" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G631" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H631" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I631" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J631" t="inlineStr">
-        <is>
-          <t>338</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>30% de desconto em serviços , alinhamento e balanceamento</t>
         </is>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>993</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>30.00%</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
@@ -36135,7 +36172,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G632" t="inlineStr">
@@ -36155,19 +36192,19 @@
       </c>
       <c r="J632" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>338</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>1442</t>
+          <t>1410</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
@@ -36187,7 +36224,7 @@
       </c>
       <c r="F633" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G633" t="inlineStr">
@@ -36207,24 +36244,24 @@
       </c>
       <c r="J633" t="inlineStr">
         <is>
-          <t>813</t>
+          <t>781</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
         <is>
-          <t>15% OFF</t>
+          <t>10%OFF</t>
         </is>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>1559</t>
+          <t>1442</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D634" t="inlineStr">
@@ -36239,12 +36276,12 @@
       </c>
       <c r="F634" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G634" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H634" t="inlineStr">
@@ -36259,24 +36296,24 @@
       </c>
       <c r="J634" t="inlineStr">
         <is>
-          <t>915</t>
+          <t>813</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nos produtos da nossa loja online.</t>
+          <t>15% OFF</t>
         </is>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>1139</t>
+          <t>1559</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
@@ -36291,12 +36328,12 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G635" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H635" t="inlineStr">
@@ -36311,24 +36348,24 @@
       </c>
       <c r="J635" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>915</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
-          <t>17% de desconto em 2024</t>
+          <t>Com este cupom você tem direito a 10% de desconto nos produtos da nossa loja online.</t>
         </is>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>1327</t>
+          <t>1139</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>17.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D636" t="inlineStr">
@@ -36343,7 +36380,7 @@
       </c>
       <c r="F636" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G636" t="inlineStr">
@@ -36363,24 +36400,24 @@
       </c>
       <c r="J636" t="inlineStr">
         <is>
-          <t>663</t>
+          <t>492</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
         <is>
-          <t>GANHE UM PROCEDIMENTO</t>
+          <t>17% de desconto em 2024</t>
         </is>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>1450</t>
+          <t>1327</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17.00%</t>
         </is>
       </c>
       <c r="D637" t="inlineStr">
@@ -36395,7 +36432,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G637" t="inlineStr">
@@ -36410,187 +36447,187 @@
       </c>
       <c r="I637" t="inlineStr">
         <is>
-          <t>2025-06-01</t>
+          <t>Sem expiracao</t>
         </is>
       </c>
       <c r="J637" t="inlineStr">
         <is>
-          <t>806</t>
+          <t>663</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
+          <t>GANHE UM PROCEDIMENTO</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>806</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 20% de desconto em todos os serviços.
 Trabalhamos com contrato de manutenção e serviços avulsos.</t>
         </is>
       </c>
-      <c r="B638" t="inlineStr">
+      <c r="B639" t="inlineStr">
         <is>
           <t>1225</t>
         </is>
       </c>
-      <c r="C638" t="inlineStr">
+      <c r="C639" t="inlineStr">
         <is>
           <t>20.00%</t>
         </is>
       </c>
-      <c r="D638" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F638" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G638" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H638" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I638" t="inlineStr">
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J638" t="inlineStr">
+      <c r="J639" t="inlineStr">
         <is>
           <t>566</t>
         </is>
       </c>
     </row>
-    <row r="639">
-      <c r="A639" t="inlineStr">
+    <row r="640">
+      <c r="A640" t="inlineStr">
         <is>
           <t>Com este cupom você tem direito a 6% de descontos em nossas peças!
 Obs: Válido para pagamento no crédito.</t>
         </is>
       </c>
-      <c r="B639" t="inlineStr">
+      <c r="B640" t="inlineStr">
         <is>
           <t>1223</t>
         </is>
       </c>
-      <c r="C639" t="inlineStr">
+      <c r="C640" t="inlineStr">
         <is>
           <t>6.00%</t>
         </is>
       </c>
-      <c r="D639" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E639" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F639" t="inlineStr">
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G639" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H639" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I639" t="inlineStr">
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J639" t="inlineStr">
+      <c r="J640" t="inlineStr">
         <is>
           <t>563</t>
-        </is>
-      </c>
-    </row>
-    <row r="640">
-      <c r="A640" t="inlineStr">
-        <is>
-          <t>15% de desconto</t>
-        </is>
-      </c>
-      <c r="B640" t="inlineStr">
-        <is>
-          <t>1072</t>
-        </is>
-      </c>
-      <c r="C640" t="inlineStr">
-        <is>
-          <t>15.00%</t>
-        </is>
-      </c>
-      <c r="D640" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E640" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F640" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G640" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H640" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I640" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J640" t="inlineStr">
-        <is>
-          <t>434</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>15% de desconto</t>
         </is>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>1586</t>
+          <t>1072</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D641" t="inlineStr">
@@ -36625,19 +36662,19 @@
       </c>
       <c r="J641" t="inlineStr">
         <is>
-          <t>941</t>
+          <t>434</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nas suas tatoos.</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>1080</t>
+          <t>1586</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -36657,7 +36694,7 @@
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G642" t="inlineStr">
@@ -36677,19 +36714,19 @@
       </c>
       <c r="J642" t="inlineStr">
         <is>
-          <t>630</t>
+          <t>941</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>10% Off</t>
+          <t>Com este cupom você tem direito a 10% de desconto nas suas tatoos.</t>
         </is>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>1342</t>
+          <t>1080</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -36709,7 +36746,7 @@
       </c>
       <c r="F643" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G643" t="inlineStr">
@@ -36729,24 +36766,24 @@
       </c>
       <c r="J643" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>630</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>20% off</t>
+          <t>10% Off</t>
         </is>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>1607</t>
+          <t>1342</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
@@ -36761,7 +36798,7 @@
       </c>
       <c r="F644" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G644" t="inlineStr">
@@ -36781,24 +36818,24 @@
       </c>
       <c r="J644" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>714</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>20% off</t>
         </is>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>1498</t>
+          <t>1607</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
@@ -36813,7 +36850,7 @@
       </c>
       <c r="F645" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G645" t="inlineStr">
@@ -36833,24 +36870,24 @@
       </c>
       <c r="J645" t="inlineStr">
         <is>
-          <t>871</t>
+          <t>959</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
         <is>
-          <t>Frete grátis nas compras acima de 50 reais.</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>1055</t>
+          <t>1498</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
@@ -36865,7 +36902,7 @@
       </c>
       <c r="F646" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G646" t="inlineStr">
@@ -36885,24 +36922,24 @@
       </c>
       <c r="J646" t="inlineStr">
         <is>
-          <t>418</t>
+          <t>871</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>Frete grátis nas compras acima de 50 reais.</t>
         </is>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>1539</t>
+          <t>1055</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D647" t="inlineStr">
@@ -36937,19 +36974,19 @@
       </c>
       <c r="J647" t="inlineStr">
         <is>
-          <t>906</t>
+          <t>418</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>1355</t>
+          <t>1539</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
@@ -36969,7 +37006,7 @@
       </c>
       <c r="F648" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G648" t="inlineStr">
@@ -36989,24 +37026,24 @@
       </c>
       <c r="J648" t="inlineStr">
         <is>
-          <t>737</t>
+          <t>906</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
         <is>
-          <t>15% de desconto ( não válido às sextas e sábados)</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>1026</t>
+          <t>1355</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D649" t="inlineStr">
@@ -37021,7 +37058,7 @@
       </c>
       <c r="F649" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G649" t="inlineStr">
@@ -37041,19 +37078,19 @@
       </c>
       <c r="J649" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>737</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t>15% de desconto nos serviços de cílios e design de sobrancelhas</t>
+          <t>15% de desconto ( não válido às sextas e sábados)</t>
         </is>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>1026</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
@@ -37073,7 +37110,7 @@
       </c>
       <c r="F650" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G650" t="inlineStr">
@@ -37093,24 +37130,24 @@
       </c>
       <c r="J650" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>361</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>A cada 1 real gasto na loja é convertido em ponto e o aluno poderá acumular ou usar de imediato.</t>
+          <t>15% de desconto nos serviços de cílios e design de sobrancelhas</t>
         </is>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>1188</t>
+          <t>995</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
@@ -37145,24 +37182,24 @@
       </c>
       <c r="J651" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>340</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>A cada 1 real gasto na loja é convertido em ponto e o aluno poderá acumular ou usar de imediato.</t>
         </is>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>1515</t>
+          <t>1188</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
@@ -37197,24 +37234,24 @@
       </c>
       <c r="J652" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>532</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>Avaliação Facial Personalizada com IA</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1515</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D653" t="inlineStr">
@@ -37229,7 +37266,7 @@
       </c>
       <c r="F653" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G653" t="inlineStr">
@@ -37249,124 +37286,124 @@
       </c>
       <c r="J653" t="inlineStr">
         <is>
-          <t>873</t>
+          <t>881</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
+          <t>Avaliação Facial Personalizada com IA</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>873</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
           <t>15% de desconto (não é válido para joias em promoção, alianças, relógios e best seller)
 Válido apenas na loja do Riomar Papicu.</t>
         </is>
       </c>
-      <c r="B654" t="inlineStr">
+      <c r="B655" t="inlineStr">
         <is>
           <t>1320</t>
         </is>
       </c>
-      <c r="C654" t="inlineStr">
+      <c r="C655" t="inlineStr">
         <is>
           <t>15.00%</t>
         </is>
       </c>
-      <c r="D654" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E654" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F654" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G654" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H654" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I654" t="inlineStr">
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J654" t="inlineStr">
+      <c r="J655" t="inlineStr">
         <is>
           <t>657</t>
-        </is>
-      </c>
-    </row>
-    <row r="655">
-      <c r="A655" t="inlineStr">
-        <is>
-          <t>10% de desconto em todos os produtos da loja. Válido apenas para pagamentos por cartão de credito.</t>
-        </is>
-      </c>
-      <c r="B655" t="inlineStr">
-        <is>
-          <t>1191</t>
-        </is>
-      </c>
-      <c r="C655" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D655" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E655" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F655" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G655" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H655" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I655" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J655" t="inlineStr">
-        <is>
-          <t>533</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" t="inlineStr">
         <is>
-          <t>10% de desconto em qualquer produto (lentes e armações)</t>
+          <t>10% de desconto em todos os produtos da loja. Válido apenas para pagamentos por cartão de credito.</t>
         </is>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>1014</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
@@ -37406,19 +37443,19 @@
       </c>
       <c r="J656" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>533</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nas suas compras.</t>
+          <t>10% de desconto em qualquer produto (lentes e armações)</t>
         </is>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>1131</t>
+          <t>1014</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -37458,66 +37495,118 @@
       </c>
       <c r="J657" t="inlineStr">
         <is>
-          <t>484</t>
+          <t>354</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto nas suas compras.</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>1131</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>484</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 20% de desconto nas compras em nossa loja.</t>
         </is>
       </c>
-      <c r="B658" t="inlineStr">
+      <c r="B659" t="inlineStr">
         <is>
           <t>1125</t>
         </is>
       </c>
-      <c r="C658" t="inlineStr">
+      <c r="C659" t="inlineStr">
         <is>
           <t>20.00%</t>
         </is>
       </c>
-      <c r="D658" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F658" t="inlineStr">
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G658" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H658" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I658" t="inlineStr">
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J658" t="inlineStr">
+      <c r="J659" t="inlineStr">
         <is>
           <t>478</t>
         </is>
       </c>
     </row>
-    <row r="660">
-      <c r="A660" t="inlineStr">
-        <is>
-          <t>Atualizado: 14/08/2026 07:46 | Ativas: 839 | Inativas: 0</t>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Atualizado: 15/08/2026 07:12 | Ativas: 840 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -37532,7 +37621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E704"/>
+  <dimension ref="A1:E705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -56298,10 +56387,35 @@
         </is>
       </c>
     </row>
-    <row r="704">
-      <c r="A704" t="inlineStr">
-        <is>
-          <t>Atualizado: 14/08/2026 07:46 | Total: 701 | c/ usuario: 186 | s/ usuario: 515</t>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>961</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Conexão Real</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Nao cadastrado</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>EVENTOS</t>
+        </is>
+      </c>
+      <c r="E703" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Atualizado: 15/08/2026 07:12 | Total: 702 | c/ usuario: 186 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -65370,7 +65484,7 @@
         </is>
       </c>
       <c r="B696" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C696" t="n">
         <v>0</v>
@@ -65379,7 +65493,7 @@
     <row r="698">
       <c r="A698" t="inlineStr">
         <is>
-          <t>Atualizado: 14/08/2026 07:46 | Total dias: 695</t>
+          <t>Atualizado: 15/08/2026 07:12 | Total dias: 695</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-16 10:16 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3110,6 +3110,43 @@
         </is>
       </c>
       <c r="G72" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>16/08/2026 07:13</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>840</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>6396</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>702</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -3483,7 +3520,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -5837,7 +5874,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -6619,7 +6656,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -9094,7 +9131,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>145</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -17767,17 +17804,17 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Cupom de 15% OFF exclusivo para alunos Green na compra de qualquer peça EUVUT!</t>
+          <t>5% de desconto nos planos Basic e Plus</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>1094</t>
+          <t>1022</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -17812,24 +17849,24 @@
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>448</t>
+          <t>359</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>5% de desconto nos planos Basic e Plus</t>
+          <t>Cupom de 15% OFF exclusivo para alunos Green na compra de qualquer peça EUVUT!</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>1022</t>
+          <t>1094</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -17844,7 +17881,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -17864,7 +17901,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>448</t>
         </is>
       </c>
     </row>
@@ -21969,7 +22006,7 @@
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -22285,7 +22322,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -22809,7 +22846,7 @@
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
@@ -24479,7 +24516,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -25837,7 +25874,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
@@ -29438,7 +29475,7 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G503" t="inlineStr">
@@ -35545,7 +35582,7 @@
       </c>
       <c r="F620" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>215</t>
         </is>
       </c>
       <c r="G620" t="inlineStr">
@@ -37318,7 +37355,7 @@
       </c>
       <c r="F654" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G654" t="inlineStr">
@@ -37606,7 +37643,7 @@
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>Atualizado: 15/08/2026 07:12 | Ativas: 840 | Inativas: 0</t>
+          <t>Atualizado: 16/08/2026 07:13 | Ativas: 840 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56415,7 +56452,7 @@
     <row r="705">
       <c r="A705" t="inlineStr">
         <is>
-          <t>Atualizado: 15/08/2026 07:12 | Total: 702 | c/ usuario: 186 | s/ usuario: 516</t>
+          <t>Atualizado: 16/08/2026 07:13 | Total: 702 | c/ usuario: 186 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -56430,7 +56467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C698"/>
+  <dimension ref="A1:C699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65490,10 +65527,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="698">
-      <c r="A698" t="inlineStr">
-        <is>
-          <t>Atualizado: 15/08/2026 07:12 | Total dias: 695</t>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>15/08/2026</t>
+        </is>
+      </c>
+      <c r="B697" t="n">
+        <v>18</v>
+      </c>
+      <c r="C697" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Atualizado: 16/08/2026 07:13 | Total dias: 696</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-17 10:24 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3147,6 +3147,43 @@
         </is>
       </c>
       <c r="G73" t="inlineStr">
+        <is>
+          <t>516</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>17/08/2026 07:21</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>840</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>6404</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>702</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
         <is>
           <t>516</t>
         </is>
@@ -9079,7 +9116,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -12069,7 +12106,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -14740,7 +14777,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -31881,7 +31918,7 @@
       </c>
       <c r="F549" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G549" t="inlineStr">
@@ -37643,7 +37680,7 @@
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>Atualizado: 16/08/2026 07:13 | Ativas: 840 | Inativas: 0</t>
+          <t>Atualizado: 17/08/2026 07:21 | Ativas: 840 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56452,7 +56489,7 @@
     <row r="705">
       <c r="A705" t="inlineStr">
         <is>
-          <t>Atualizado: 16/08/2026 07:13 | Total: 702 | c/ usuario: 186 | s/ usuario: 516</t>
+          <t>Atualizado: 17/08/2026 07:21 | Total: 702 | c/ usuario: 186 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -56467,7 +56504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C699"/>
+  <dimension ref="A1:C701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65540,10 +65577,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>16/08/2026</t>
+        </is>
+      </c>
+      <c r="B698" t="n">
+        <v>6</v>
+      </c>
+      <c r="C698" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="699">
       <c r="A699" t="inlineStr">
         <is>
-          <t>Atualizado: 16/08/2026 07:13 | Total dias: 696</t>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B699" t="n">
+        <v>2</v>
+      </c>
+      <c r="C699" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Atualizado: 17/08/2026 07:21 | Total dias: 698</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-21 10:22 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3295,6 +3295,43 @@
         </is>
       </c>
       <c r="G77" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>21/08/2026 07:19</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>843</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>6420</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -12009,7 +12046,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -17559,7 +17596,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -17715,7 +17752,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
@@ -24507,7 +24544,7 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -24768,7 +24805,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>64</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -28215,7 +28252,7 @@
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G476" t="inlineStr">
@@ -29728,7 +29765,7 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="G505" t="inlineStr">
@@ -37843,7 +37880,7 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>Atualizado: 20/08/2026 07:19 | Ativas: 843 | Inativas: 0</t>
+          <t>Atualizado: 21/08/2026 07:19 | Ativas: 843 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56679,7 +56716,7 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>Atualizado: 20/08/2026 07:19 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
+          <t>Atualizado: 21/08/2026 07:19 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -56694,7 +56731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C704"/>
+  <dimension ref="A1:C705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65826,16 +65863,29 @@
         </is>
       </c>
       <c r="B702" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C702" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="704">
-      <c r="A704" t="inlineStr">
-        <is>
-          <t>Atualizado: 20/08/2026 07:19 | Total dias: 701</t>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="B703" t="n">
+        <v>1</v>
+      </c>
+      <c r="C703" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Atualizado: 21/08/2026 07:19 | Total dias: 702</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-22 10:15 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3332,6 +3332,43 @@
         </is>
       </c>
       <c r="G78" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>22/08/2026 07:12</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>843</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>6425</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -11729,7 +11766,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -35715,7 +35752,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G619" t="inlineStr">
@@ -37176,7 +37213,7 @@
       </c>
       <c r="F647" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G647" t="inlineStr">
@@ -37880,7 +37917,7 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>Atualizado: 21/08/2026 07:19 | Ativas: 843 | Inativas: 0</t>
+          <t>Atualizado: 22/08/2026 07:12 | Ativas: 843 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56716,7 +56753,7 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>Atualizado: 21/08/2026 07:19 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
+          <t>Atualizado: 22/08/2026 07:12 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -56731,7 +56768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C705"/>
+  <dimension ref="A1:C706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65876,16 +65913,29 @@
         </is>
       </c>
       <c r="B703" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C703" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="705">
-      <c r="A705" t="inlineStr">
-        <is>
-          <t>Atualizado: 21/08/2026 07:19 | Total dias: 702</t>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
+        </is>
+      </c>
+      <c r="B704" t="n">
+        <v>1</v>
+      </c>
+      <c r="C704" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Atualizado: 22/08/2026 07:12 | Total dias: 703</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-23 10:18 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3369,6 +3369,43 @@
         </is>
       </c>
       <c r="G79" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>23/08/2026 07:14</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>843</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>6427</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -37917,7 +37954,7 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>Atualizado: 22/08/2026 07:12 | Ativas: 843 | Inativas: 0</t>
+          <t>Atualizado: 23/08/2026 07:14 | Ativas: 843 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56753,7 +56790,7 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>Atualizado: 22/08/2026 07:12 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
+          <t>Atualizado: 23/08/2026 07:14 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -65926,7 +65963,7 @@
         </is>
       </c>
       <c r="B704" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C704" t="n">
         <v>0</v>
@@ -65935,7 +65972,7 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>Atualizado: 22/08/2026 07:12 | Total dias: 703</t>
+          <t>Atualizado: 23/08/2026 07:14 | Total dias: 703</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-24 10:30 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3406,6 +3406,43 @@
         </is>
       </c>
       <c r="G80" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>24/08/2026 07:27</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>843</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>6430</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -9442,7 +9479,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -12120,7 +12157,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>95</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -35109,7 +35146,7 @@
       </c>
       <c r="F606" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>68</t>
         </is>
       </c>
       <c r="G606" t="inlineStr">
@@ -37954,7 +37991,7 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>Atualizado: 23/08/2026 07:14 | Ativas: 843 | Inativas: 0</t>
+          <t>Atualizado: 24/08/2026 07:27 | Ativas: 843 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56790,7 +56827,7 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>Atualizado: 23/08/2026 07:14 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
+          <t>Atualizado: 24/08/2026 07:27 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -56805,7 +56842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C706"/>
+  <dimension ref="A1:C707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65969,10 +66006,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="706">
-      <c r="A706" t="inlineStr">
-        <is>
-          <t>Atualizado: 23/08/2026 07:14 | Total dias: 703</t>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
+      <c r="B705" t="n">
+        <v>3</v>
+      </c>
+      <c r="C705" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Atualizado: 24/08/2026 07:27 | Total dias: 704</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-25 10:26 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3443,6 +3443,43 @@
         </is>
       </c>
       <c r="G81" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>25/08/2026 07:23</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>843</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>6440</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -7428,7 +7465,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -23194,7 +23231,7 @@
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>82</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
@@ -35930,7 +35967,7 @@
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>221</t>
         </is>
       </c>
       <c r="G621" t="inlineStr">
@@ -37991,7 +38028,7 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>Atualizado: 24/08/2026 07:27 | Ativas: 843 | Inativas: 0</t>
+          <t>Atualizado: 25/08/2026 07:23 | Ativas: 843 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56827,7 +56864,7 @@
     <row r="706">
       <c r="A706" t="inlineStr">
         <is>
-          <t>Atualizado: 24/08/2026 07:27 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
+          <t>Atualizado: 25/08/2026 07:23 | Total: 703 | c/ usuario: 189 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -56842,7 +56879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C707"/>
+  <dimension ref="A1:C709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66019,10 +66056,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="B706" t="n">
+        <v>9</v>
+      </c>
+      <c r="C706" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="707">
       <c r="A707" t="inlineStr">
         <is>
-          <t>Atualizado: 24/08/2026 07:27 | Total dias: 704</t>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="B707" t="n">
+        <v>1</v>
+      </c>
+      <c r="C707" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Atualizado: 25/08/2026 07:23 | Total dias: 706</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-27 20:10 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3517,6 +3517,43 @@
         </is>
       </c>
       <c r="G83" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>27/08/2026 17:06</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>843</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>6417</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>704</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -7341,7 +7378,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>378</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -7448,7 +7485,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -8238,7 +8275,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -10234,7 +10271,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>145</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -12283,7 +12320,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>149</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -15056,7 +15093,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -35273,7 +35310,7 @@
       </c>
       <c r="F607" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70</t>
         </is>
       </c>
       <c r="G607" t="inlineStr">
@@ -37570,7 +37607,7 @@
       </c>
       <c r="F651" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G651" t="inlineStr">
@@ -38066,7 +38103,7 @@
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>Atualizado: 26/08/2026 07:25 | Ativas: 843 | Inativas: 0</t>
+          <t>Atualizado: 27/08/2026 17:06 | Ativas: 843 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -56927,7 +56964,7 @@
     <row r="707">
       <c r="A707" t="inlineStr">
         <is>
-          <t>Atualizado: 26/08/2026 07:25 | Total: 704 | c/ usuario: 190 | s/ usuario: 514</t>
+          <t>Atualizado: 27/08/2026 17:06 | Total: 704 | c/ usuario: 190 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -56942,7 +56979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C710"/>
+  <dimension ref="A1:C711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66152,16 +66189,29 @@
         </is>
       </c>
       <c r="B708" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C708" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="710">
-      <c r="A710" t="inlineStr">
-        <is>
-          <t>Atualizado: 26/08/2026 07:25 | Total dias: 707</t>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B709" t="n">
+        <v>14</v>
+      </c>
+      <c r="C709" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Atualizado: 27/08/2026 17:06 | Total dias: 708</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-29 14:50 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3591,6 +3591,43 @@
         </is>
       </c>
       <c r="G85" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>29/08/2026 11:47</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>6424</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -28670,7 +28707,7 @@
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G479" t="inlineStr">
@@ -32430,7 +32467,7 @@
       </c>
       <c r="F551" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G551" t="inlineStr">
@@ -38194,7 +38231,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 28/08/2026 18:03 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 29/08/2026 11:47 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57082,7 +57119,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 28/08/2026 18:03 | Total: 705 | c/ usuario: 190 | s/ usuario: 515</t>
+          <t>Atualizado: 29/08/2026 11:47 | Total: 705 | c/ usuario: 190 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -57097,7 +57134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C712"/>
+  <dimension ref="A1:C713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66339,10 +66376,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="712">
-      <c r="A712" t="inlineStr">
-        <is>
-          <t>Atualizado: 28/08/2026 18:03 | Total dias: 709</t>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="B711" t="n">
+        <v>2</v>
+      </c>
+      <c r="C711" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Atualizado: 29/08/2026 11:47 | Total dias: 710</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-08-30 14:40 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3628,6 +3628,43 @@
         </is>
       </c>
       <c r="G86" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>30/08/2026 11:36</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>6433</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -4633,7 +4670,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -9664,7 +9701,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -28655,7 +28692,7 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>58</t>
         </is>
       </c>
       <c r="G478" t="inlineStr">
@@ -30637,7 +30674,7 @@
       </c>
       <c r="F516" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G516" t="inlineStr">
@@ -36222,7 +36259,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>223</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38231,7 +38268,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 29/08/2026 11:47 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 30/08/2026 11:36 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57119,7 +57156,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 29/08/2026 11:47 | Total: 705 | c/ usuario: 190 | s/ usuario: 515</t>
+          <t>Atualizado: 30/08/2026 11:36 | Total: 705 | c/ usuario: 190 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -66383,7 +66420,7 @@
         </is>
       </c>
       <c r="B711" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C711" t="n">
         <v>0</v>
@@ -66392,7 +66429,7 @@
     <row r="713">
       <c r="A713" t="inlineStr">
         <is>
-          <t>Atualizado: 29/08/2026 11:47 | Total dias: 710</t>
+          <t>Atualizado: 30/08/2026 11:36 | Total dias: 710</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-04 13:57 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3667,6 +3667,43 @@
       <c r="G87" t="inlineStr">
         <is>
           <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>04/09/2026 10:54</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>6469</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>514</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4179,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4247,7 +4284,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5609,7 +5646,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -6235,7 +6272,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -12272,7 +12309,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -12379,7 +12416,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>96</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -12431,7 +12468,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -14729,7 +14766,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -18453,7 +18490,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -19754,7 +19791,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -20230,7 +20267,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -23575,7 +23612,7 @@
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
@@ -24723,7 +24760,7 @@
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
@@ -26760,7 +26797,7 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
@@ -27593,7 +27630,7 @@
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G457" t="inlineStr">
@@ -28692,7 +28729,7 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>59</t>
         </is>
       </c>
       <c r="G478" t="inlineStr">
@@ -31617,7 +31654,7 @@
       </c>
       <c r="F534" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G534" t="inlineStr">
@@ -33026,7 +33063,7 @@
       </c>
       <c r="F561" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G561" t="inlineStr">
@@ -33182,7 +33219,7 @@
       </c>
       <c r="F564" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G564" t="inlineStr">
@@ -36259,7 +36296,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>227</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38268,7 +38305,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 30/08/2026 11:36 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 04/09/2026 10:54 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57139,7 +57176,7 @@
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>Nao cadastrado</t>
+          <t>Jéssica Ferratoni / marketing@nutrafit.com.br</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
@@ -57156,7 +57193,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 30/08/2026 11:36 | Total: 705 | c/ usuario: 190 | s/ usuario: 515</t>
+          <t>Atualizado: 04/09/2026 10:54 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57171,7 +57208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C713"/>
+  <dimension ref="A1:C719"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66426,10 +66463,88 @@
         <v>0</v>
       </c>
     </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="B712" t="n">
+        <v>1</v>
+      </c>
+      <c r="C712" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="713">
       <c r="A713" t="inlineStr">
         <is>
-          <t>Atualizado: 30/08/2026 11:36 | Total dias: 710</t>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="B713" t="n">
+        <v>3</v>
+      </c>
+      <c r="C713" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="B714" t="n">
+        <v>6</v>
+      </c>
+      <c r="C714" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B715" t="n">
+        <v>12</v>
+      </c>
+      <c r="C715" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="B716" t="n">
+        <v>12</v>
+      </c>
+      <c r="C716" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B717" t="n">
+        <v>2</v>
+      </c>
+      <c r="C717" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Atualizado: 04/09/2026 10:54 | Total dias: 716</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-05 13:11 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3702,6 +3702,43 @@
         </is>
       </c>
       <c r="G88" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>05/09/2026 10:09</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>6474</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -6793,7 +6830,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -7526,7 +7563,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>378</t>
+          <t>379</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -12468,7 +12505,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>151</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -38305,7 +38342,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 04/09/2026 10:54 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 05/09/2026 10:09 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57193,7 +57230,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 04/09/2026 10:54 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 05/09/2026 10:09 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57208,7 +57245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C719"/>
+  <dimension ref="A1:C720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66535,16 +66572,29 @@
         </is>
       </c>
       <c r="B717" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C717" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="719">
-      <c r="A719" t="inlineStr">
-        <is>
-          <t>Atualizado: 04/09/2026 10:54 | Total dias: 716</t>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="B718" t="n">
+        <v>1</v>
+      </c>
+      <c r="C718" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Atualizado: 05/09/2026 10:09 | Total dias: 717</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-06 13:19 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3739,6 +3739,43 @@
         </is>
       </c>
       <c r="G89" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>06/09/2026 10:17</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>6481</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -5683,7 +5720,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7563,7 +7600,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>380</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -12136,7 +12173,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -22287,7 +22324,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
@@ -36333,7 +36370,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>228</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -37064,7 +37101,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G637" t="inlineStr">
@@ -38342,7 +38379,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 05/09/2026 10:09 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 06/09/2026 10:17 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57230,7 +57267,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 05/09/2026 10:09 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 06/09/2026 10:17 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -66585,7 +66622,7 @@
         </is>
       </c>
       <c r="B718" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C718" t="n">
         <v>0</v>
@@ -66594,7 +66631,7 @@
     <row r="720">
       <c r="A720" t="inlineStr">
         <is>
-          <t>Atualizado: 05/09/2026 10:09 | Total dias: 717</t>
+          <t>Atualizado: 06/09/2026 10:17 | Total dias: 717</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-07 15:27 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3776,6 +3776,43 @@
         </is>
       </c>
       <c r="G90" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>07/09/2026 12:25</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>6484</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -32721,7 +32758,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G553" t="inlineStr">
@@ -34074,7 +34111,7 @@
       </c>
       <c r="F579" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G579" t="inlineStr">
@@ -38379,7 +38416,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 06/09/2026 10:17 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 07/09/2026 12:25 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57267,7 +57304,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 06/09/2026 10:17 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 07/09/2026 12:25 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57282,7 +57319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C720"/>
+  <dimension ref="A1:C721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66628,10 +66665,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="720">
-      <c r="A720" t="inlineStr">
-        <is>
-          <t>Atualizado: 06/09/2026 10:17 | Total dias: 717</t>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="B719" t="n">
+        <v>3</v>
+      </c>
+      <c r="C719" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Atualizado: 07/09/2026 12:25 | Total dias: 718</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-08 14:00 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3813,6 +3813,43 @@
         </is>
       </c>
       <c r="G91" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08/09/2026 10:58</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>6487</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -6383,7 +6420,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>144</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -36407,7 +36444,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>229</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38416,7 +38453,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 07/09/2026 12:25 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 08/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57304,7 +57341,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 07/09/2026 12:25 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 08/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57319,7 +57356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C721"/>
+  <dimension ref="A1:C722"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66678,10 +66715,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="721">
-      <c r="A721" t="inlineStr">
-        <is>
-          <t>Atualizado: 07/09/2026 12:25 | Total dias: 718</t>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B720" t="n">
+        <v>3</v>
+      </c>
+      <c r="C720" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Atualizado: 08/09/2026 10:58 | Total dias: 719</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-09 14:05 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3850,6 +3850,43 @@
         </is>
       </c>
       <c r="G92" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>09/09/2026 11:03</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>6493</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -9834,7 +9871,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -10936,7 +10973,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -25430,7 +25467,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -36234,7 +36271,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G619" t="inlineStr">
@@ -36444,7 +36481,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>230</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38453,7 +38490,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 08/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 09/09/2026 11:03 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57341,7 +57378,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 08/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 09/09/2026 11:03 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57356,7 +57393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C722"/>
+  <dimension ref="A1:C724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66728,10 +66765,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B721" t="n">
+        <v>4</v>
+      </c>
+      <c r="C721" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="722">
       <c r="A722" t="inlineStr">
         <is>
-          <t>Atualizado: 08/09/2026 10:58 | Total dias: 719</t>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B722" t="n">
+        <v>2</v>
+      </c>
+      <c r="C722" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Atualizado: 09/09/2026 11:03 | Total dias: 721</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-10 13:59 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3887,6 +3887,43 @@
         </is>
       </c>
       <c r="G93" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>10/09/2026 10:58</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>6505</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -5206,7 +5243,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7711,7 +7748,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>381</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -14741,7 +14778,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -16106,7 +16143,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -25571,7 +25608,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>65</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -28914,7 +28951,7 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>60</t>
         </is>
       </c>
       <c r="G478" t="inlineStr">
@@ -32313,7 +32350,7 @@
       </c>
       <c r="F543" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G543" t="inlineStr">
@@ -36481,7 +36518,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>231</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -36951,7 +36988,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G632" t="inlineStr">
@@ -38490,7 +38527,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 09/09/2026 11:03 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 10/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57378,7 +57415,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 09/09/2026 11:03 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 10/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57393,7 +57430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C724"/>
+  <dimension ref="A1:C725"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66785,16 +66822,29 @@
         </is>
       </c>
       <c r="B722" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C722" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="724">
-      <c r="A724" t="inlineStr">
-        <is>
-          <t>Atualizado: 09/09/2026 11:03 | Total dias: 721</t>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B723" t="n">
+        <v>1</v>
+      </c>
+      <c r="C723" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Atualizado: 10/09/2026 10:58 | Total dias: 722</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-11 14:00 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3924,6 +3924,43 @@
         </is>
       </c>
       <c r="G94" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>11/09/2026 10:58</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>6507</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -30150,7 +30187,7 @@
       </c>
       <c r="F501" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G501" t="inlineStr">
@@ -38527,7 +38564,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 10/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 11/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57415,7 +57452,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 10/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 11/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -66835,7 +66872,7 @@
         </is>
       </c>
       <c r="B723" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C723" t="n">
         <v>0</v>
@@ -66844,7 +66881,7 @@
     <row r="725">
       <c r="A725" t="inlineStr">
         <is>
-          <t>Atualizado: 10/09/2026 10:58 | Total dias: 722</t>
+          <t>Atualizado: 11/09/2026 10:58 | Total dias: 722</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-12 13:16 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3961,6 +3961,43 @@
         </is>
       </c>
       <c r="G95" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>12/09/2026 10:14</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>6513</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -7470,7 +7507,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -8789,7 +8826,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -15606,7 +15643,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -19530,7 +19567,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -30970,7 +31007,7 @@
       </c>
       <c r="F516" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G516" t="inlineStr">
@@ -33010,7 +33047,7 @@
       </c>
       <c r="F555" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G555" t="inlineStr">
@@ -38564,7 +38601,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 11/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 12/09/2026 10:14 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57452,7 +57489,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 11/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 12/09/2026 10:14 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57467,7 +57504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C725"/>
+  <dimension ref="A1:C727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66878,10 +66915,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B724" t="n">
+        <v>4</v>
+      </c>
+      <c r="C724" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="725">
       <c r="A725" t="inlineStr">
         <is>
-          <t>Atualizado: 11/09/2026 10:58 | Total dias: 722</t>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="B725" t="n">
+        <v>2</v>
+      </c>
+      <c r="C725" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Atualizado: 12/09/2026 10:14 | Total dias: 724</t>
         </is>
       </c>
     </row>

</xml_diff>